<commit_message>
Itinerario V1.0.1 y Cronograma V1.0.0
</commit_message>
<xml_diff>
--- a/Cronograma/Itinerario _PPP_V1.xlsx
+++ b/Cronograma/Itinerario _PPP_V1.xlsx
@@ -281,7 +281,7 @@
     <t xml:space="preserve">Ajustar eventos, validaciones y comportamientos ejecutados del lado del cliente.</t>
   </si>
   <si>
-    <t xml:space="preserve">Configurar funciones relacionadas con actualizaciones AJAX, calendarios y componentes interactivos.</t>
+    <t xml:space="preserve">Configurar funciones relacionadas con actualizaciones, calendarios y componentes interactivos.</t>
   </si>
   <si>
     <t xml:space="preserve">Adaptación de componentes XHTML</t>
@@ -305,7 +305,7 @@
     <t xml:space="preserve">Corregir inconsistencias de estilos, eventos JavaScript y distribución de componentes.</t>
   </si>
   <si>
-    <t xml:space="preserve">Verificar la navegación y documentar los cambios realizados en el frontend.</t>
+    <t xml:space="preserve">Verificar la navegación y el comportamiento de los componentes interactivos de las vistas.</t>
   </si>
   <si>
     <t xml:space="preserve">Análisis del sistema ComercializadorasCLDH</t>
@@ -317,7 +317,7 @@
     <t xml:space="preserve">Identificar los procesos que deben mantenerse en la futura plataforma web.</t>
   </si>
   <si>
-    <t xml:space="preserve">Registrar las funcionalidades que requieren adaptación o mejora durante la migración.</t>
+    <t xml:space="preserve">Determinar las principales funcionalidades que serán consideradas durante la migración.</t>
   </si>
   <si>
     <t xml:space="preserve">Definición de la arquitectura web</t>
@@ -350,10 +350,10 @@
     <t xml:space="preserve">Analizar las funcionalidades y flujo de trabajo del sistema de escritorio a partir de las capturas e información proporcionadas.</t>
   </si>
   <si>
-    <t xml:space="preserve">Definir las funcionalidades que serán desarrolladas inicialmente en la plataforma web.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Identificar los componentes y procesos que deberán ser adaptados durante el proceso de migración.</t>
+    <t xml:space="preserve">Establecer el alcance inicial de la plataforma web a partir de las funcionalidades identificadas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Definir los componentes del sistema que deberán ser adaptados durante el proceso de migración.</t>
   </si>
   <si>
     <t xml:space="preserve">Revisión de la estructura de datos</t>
@@ -638,7 +638,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="45">
+  <borders count="27">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -793,31 +793,7 @@
       <top style="thin">
         <color theme="1"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="none"/>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
+      <bottom style="none"/>
       <diagonal style="none"/>
     </border>
     <border>
@@ -827,19 +803,6 @@
       <right style="thin">
         <color theme="1"/>
       </right>
-      <top/>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
       <top style="none"/>
       <bottom style="none"/>
       <diagonal style="none"/>
@@ -848,69 +811,12 @@
       <left style="thin">
         <color auto="1"/>
       </left>
-      <right style="none"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top style="none"/>
       <bottom style="thin">
         <color theme="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="thin">
-        <color auto="1"/>
       </bottom>
       <diagonal style="none"/>
     </border>
@@ -934,10 +840,8 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top style="thin">
-        <color theme="1"/>
-      </top>
-      <bottom/>
+      <top style="none"/>
+      <bottom style="none"/>
       <diagonal style="none"/>
     </border>
     <border>
@@ -945,30 +849,6 @@
         <color auto="1"/>
       </left>
       <right style="none"/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
       <top style="none"/>
       <bottom style="thin">
         <color theme="1"/>
@@ -979,47 +859,34 @@
       <left style="thin">
         <color auto="1"/>
       </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
+      <right style="none"/>
+      <top style="none"/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left style="thin">
         <color theme="1"/>
       </left>
       <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
         <color theme="1"/>
+      </top>
+      <bottom style="none"/>
+      <diagonal style="none"/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
       </right>
-      <top/>
+      <top style="none"/>
       <bottom style="thin">
         <color theme="1"/>
       </bottom>
@@ -1032,81 +899,10 @@
       <right style="thin">
         <color auto="1"/>
       </right>
-      <top/>
+      <top style="none"/>
       <bottom style="thin">
         <color auto="1"/>
       </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="none"/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="none"/>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="none"/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="none"/>
-      <top/>
-      <bottom/>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="none"/>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top/>
-      <bottom style="none"/>
       <diagonal style="none"/>
     </border>
     <border>
@@ -1176,7 +972,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="84">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1205,9 +1001,6 @@
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf fontId="2" fillId="2" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1227,9 +1020,6 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="3" borderId="5" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="5" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="3" borderId="4" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1259,179 +1049,98 @@
     <xf fontId="0" fillId="0" borderId="5" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="11" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="12" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="8" numFmtId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="11" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="8" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="9" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="13" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="10" numFmtId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="14" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="15" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="3" borderId="16" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="4" borderId="12" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="4" borderId="13" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="3" borderId="17" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="4" borderId="15" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="5" numFmtId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="18" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="3" borderId="5" numFmtId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="3" borderId="19" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="3" borderId="20" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="3" borderId="18" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="10" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="3" borderId="12" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="3" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="3" borderId="10" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="3" fillId="3" borderId="15" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="3" borderId="21" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="5" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="11" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="6" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="12" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="8" numFmtId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="11" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="8" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="9" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="13" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="10" numFmtId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="14" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="15" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="16" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="4" borderId="12" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="4" borderId="13" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="17" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="4" borderId="15" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="5" numFmtId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="18" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="19" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="20" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="21" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="22" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="23" numFmtId="164" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="5" numFmtId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="24" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="25" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="4" borderId="19" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="26" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="4" borderId="21" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="27" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="22" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="4" borderId="23" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="8" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="25" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="10" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="28" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="3" borderId="19" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="29" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="0" numFmtId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf fontId="0" fillId="3" borderId="5" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="30" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="3" fillId="3" borderId="31" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="28" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="29" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="32" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="33" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="34" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="5" numFmtId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="35" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="33" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="3" borderId="34" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="35" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="36" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="37" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="30" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="38" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="5" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1439,36 +1148,15 @@
     <xf fontId="0" fillId="4" borderId="5" numFmtId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="4" borderId="5" numFmtId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf fontId="0" fillId="4" borderId="5" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="5" numFmtId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf fontId="0" fillId="4" borderId="5" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="4" borderId="5" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="4" borderId="5" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="4" numFmtId="14" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="5" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="5" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="5" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf fontId="0" fillId="4" borderId="4" numFmtId="14" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1496,15 +1184,9 @@
     <xf fontId="0" fillId="4" borderId="10" numFmtId="165" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="4" borderId="39" numFmtId="164" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" textRotation="255" vertical="top" wrapText="1"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="4" numFmtId="165" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="5" numFmtId="165" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1523,22 +1205,22 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="40" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="22" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="5" borderId="41" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="5" borderId="23" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="42" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="24" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="5" borderId="43" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="5" borderId="25" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="44" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="26" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="44" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="26" numFmtId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2084,7 +1766,7 @@
       <c r="A5" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="4" t="s">
         <v>8</v>
       </c>
     </row>
@@ -2098,2152 +1780,2152 @@
     </row>
     <row r="7" ht="24.75" customHeight="1"/>
     <row r="8" ht="52.5" customHeight="1">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="D8" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="12"/>
-      <c r="F8" s="11" t="s">
+      <c r="E8" s="11"/>
+      <c r="F8" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="G8" s="13" t="s">
+      <c r="G8" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="H8" s="14" t="s">
+      <c r="H8" s="13" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="9" ht="52.5" customHeight="1">
-      <c r="A9" s="15">
+      <c r="A9" s="14">
         <v>46274</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="17">
+      <c r="D9" s="15">
         <v>3</v>
       </c>
-      <c r="E9" s="18"/>
-      <c r="F9" s="19" t="s">
+      <c r="E9" s="16"/>
+      <c r="F9" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="G9" s="20">
-        <v>6</v>
-      </c>
-      <c r="H9" s="21"/>
+      <c r="G9" s="18">
+        <v>6</v>
+      </c>
+      <c r="H9" s="19"/>
     </row>
     <row r="10" ht="46.5" customHeight="1">
-      <c r="A10" s="22"/>
-      <c r="B10" s="22"/>
-      <c r="C10" s="16" t="s">
+      <c r="A10" s="20"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="17">
-        <v>2</v>
-      </c>
-      <c r="E10" s="18"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="24"/>
-      <c r="H10" s="21"/>
+      <c r="D10" s="15">
+        <v>2</v>
+      </c>
+      <c r="E10" s="16"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="19"/>
     </row>
     <row r="11" ht="28.5">
-      <c r="A11" s="25"/>
-      <c r="B11" s="25"/>
-      <c r="C11" s="16" t="s">
+      <c r="A11" s="23"/>
+      <c r="B11" s="23"/>
+      <c r="C11" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="17">
+      <c r="D11" s="15">
         <v>1</v>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="16">
         <f>SUM(D9:D11)</f>
         <v>6</v>
       </c>
-      <c r="F11" s="23"/>
-      <c r="G11" s="24"/>
-      <c r="H11" s="21"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="19"/>
     </row>
     <row r="12" ht="28.5">
-      <c r="A12" s="26">
+      <c r="A12" s="24">
         <v>46275</v>
       </c>
-      <c r="B12" s="26" t="s">
+      <c r="B12" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="C12" s="27" t="s">
+      <c r="C12" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="28">
-        <v>2</v>
-      </c>
-      <c r="E12" s="29"/>
-      <c r="F12" s="30" t="s">
+      <c r="D12" s="25">
+        <v>2</v>
+      </c>
+      <c r="E12" s="26"/>
+      <c r="F12" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="G12" s="31">
-        <v>6</v>
-      </c>
-      <c r="H12" s="32"/>
+      <c r="G12" s="28">
+        <v>6</v>
+      </c>
+      <c r="H12" s="29"/>
     </row>
     <row r="13" ht="28.5">
-      <c r="A13" s="33"/>
-      <c r="B13" s="33"/>
-      <c r="C13" s="27" t="s">
+      <c r="A13" s="30"/>
+      <c r="B13" s="30"/>
+      <c r="C13" s="25" t="s">
         <v>25</v>
       </c>
-      <c r="D13" s="28">
-        <v>2</v>
-      </c>
-      <c r="E13" s="34"/>
-      <c r="F13" s="35"/>
-      <c r="G13" s="36"/>
-      <c r="H13" s="37"/>
+      <c r="D13" s="25">
+        <v>2</v>
+      </c>
+      <c r="E13" s="31"/>
+      <c r="F13" s="32"/>
+      <c r="G13" s="33"/>
+      <c r="H13" s="34"/>
     </row>
     <row r="14" ht="42.75">
-      <c r="A14" s="38"/>
-      <c r="B14" s="38"/>
-      <c r="C14" s="27" t="s">
+      <c r="A14" s="35"/>
+      <c r="B14" s="35"/>
+      <c r="C14" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="D14" s="28">
-        <v>2</v>
-      </c>
-      <c r="E14" s="34">
+      <c r="D14" s="25">
+        <v>2</v>
+      </c>
+      <c r="E14" s="31">
         <f>SUM(D12:D14)</f>
         <v>6</v>
       </c>
-      <c r="F14" s="39"/>
-      <c r="G14" s="36"/>
-      <c r="H14" s="40"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="33"/>
+      <c r="H14" s="37"/>
     </row>
     <row r="15" ht="42.75">
-      <c r="A15" s="15">
+      <c r="A15" s="14">
         <v>46276</v>
       </c>
-      <c r="B15" s="15" t="s">
+      <c r="B15" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="16" t="s">
+      <c r="C15" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="17">
-        <v>2</v>
-      </c>
-      <c r="E15" s="18"/>
-      <c r="F15" s="41" t="s">
+      <c r="D15" s="15">
+        <v>2</v>
+      </c>
+      <c r="E15" s="16"/>
+      <c r="F15" s="38" t="s">
         <v>20</v>
       </c>
-      <c r="G15" s="20">
-        <v>6</v>
-      </c>
-      <c r="H15" s="42"/>
+      <c r="G15" s="18">
+        <v>6</v>
+      </c>
+      <c r="H15" s="39"/>
     </row>
     <row r="16" ht="28.5">
-      <c r="A16" s="22"/>
-      <c r="B16" s="22"/>
-      <c r="C16" s="16" t="s">
+      <c r="A16" s="20"/>
+      <c r="B16" s="20"/>
+      <c r="C16" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="17">
-        <v>2</v>
-      </c>
-      <c r="E16" s="18"/>
-      <c r="F16" s="41"/>
-      <c r="G16" s="24"/>
-      <c r="H16" s="43"/>
+      <c r="D16" s="15">
+        <v>2</v>
+      </c>
+      <c r="E16" s="16"/>
+      <c r="F16" s="38"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="40"/>
     </row>
     <row r="17" ht="28.5">
-      <c r="A17" s="25"/>
-      <c r="B17" s="25"/>
-      <c r="C17" s="16" t="s">
+      <c r="A17" s="23"/>
+      <c r="B17" s="23"/>
+      <c r="C17" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="17">
-        <v>2</v>
-      </c>
-      <c r="E17" s="18">
+      <c r="D17" s="15">
+        <v>2</v>
+      </c>
+      <c r="E17" s="16">
         <f>SUM(D15:D17)</f>
         <v>6</v>
       </c>
-      <c r="F17" s="41"/>
-      <c r="G17" s="44"/>
-      <c r="H17" s="45"/>
+      <c r="F17" s="38"/>
+      <c r="G17" s="41"/>
+      <c r="H17" s="42"/>
     </row>
     <row r="18" ht="28.5">
-      <c r="A18" s="46">
+      <c r="A18" s="43">
         <v>46279</v>
       </c>
-      <c r="B18" s="46" t="s">
+      <c r="B18" s="43" t="s">
         <v>31</v>
       </c>
-      <c r="C18" s="27" t="s">
+      <c r="C18" s="25" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="28">
+      <c r="D18" s="25">
         <v>1</v>
       </c>
-      <c r="E18" s="29"/>
-      <c r="F18" s="47" t="s">
+      <c r="E18" s="26"/>
+      <c r="F18" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="G18" s="36">
-        <v>6</v>
-      </c>
-      <c r="H18" s="48"/>
+      <c r="G18" s="33">
+        <v>6</v>
+      </c>
+      <c r="H18" s="29"/>
     </row>
     <row r="19" ht="28.5">
-      <c r="A19" s="46"/>
-      <c r="B19" s="46"/>
-      <c r="C19" s="28" t="s">
+      <c r="A19" s="43"/>
+      <c r="B19" s="43"/>
+      <c r="C19" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="D19" s="28">
-        <v>2</v>
-      </c>
-      <c r="E19" s="34"/>
-      <c r="F19" s="49"/>
-      <c r="G19" s="36"/>
-      <c r="H19" s="50"/>
+      <c r="D19" s="25">
+        <v>2</v>
+      </c>
+      <c r="E19" s="31"/>
+      <c r="F19" s="32"/>
+      <c r="G19" s="33"/>
+      <c r="H19" s="34"/>
     </row>
     <row r="20">
-      <c r="A20" s="46"/>
-      <c r="B20" s="46"/>
-      <c r="C20" s="28" t="s">
+      <c r="A20" s="43"/>
+      <c r="B20" s="43"/>
+      <c r="C20" s="25" t="s">
         <v>34</v>
       </c>
-      <c r="D20" s="28">
+      <c r="D20" s="25">
         <v>3</v>
       </c>
-      <c r="E20" s="34">
+      <c r="E20" s="31">
         <f>SUM(D18:D20)</f>
         <v>6</v>
       </c>
-      <c r="F20" s="39"/>
-      <c r="G20" s="51"/>
-      <c r="H20" s="52"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="44"/>
+      <c r="H20" s="37"/>
     </row>
     <row r="21" ht="28.5">
-      <c r="A21" s="53">
+      <c r="A21" s="45">
         <v>46280</v>
       </c>
-      <c r="B21" s="53" t="s">
+      <c r="B21" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="C21" s="17" t="s">
+      <c r="C21" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="D21" s="17">
-        <v>2</v>
-      </c>
-      <c r="E21" s="18"/>
-      <c r="F21" s="54" t="s">
+      <c r="D21" s="15">
+        <v>2</v>
+      </c>
+      <c r="E21" s="16"/>
+      <c r="F21" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="G21" s="55">
-        <v>6</v>
-      </c>
-      <c r="H21" s="56"/>
+      <c r="G21" s="18">
+        <v>6</v>
+      </c>
+      <c r="H21" s="39"/>
     </row>
     <row r="22">
-      <c r="A22" s="53"/>
-      <c r="B22" s="53"/>
-      <c r="C22" s="17" t="s">
+      <c r="A22" s="45"/>
+      <c r="B22" s="45"/>
+      <c r="C22" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="D22" s="17">
+      <c r="D22" s="15">
         <v>1</v>
       </c>
-      <c r="E22" s="18"/>
-      <c r="F22" s="57"/>
-      <c r="G22" s="24"/>
-      <c r="H22" s="58"/>
+      <c r="E22" s="16"/>
+      <c r="F22" s="38"/>
+      <c r="G22" s="22"/>
+      <c r="H22" s="40"/>
     </row>
     <row r="23">
-      <c r="A23" s="53"/>
-      <c r="B23" s="53"/>
-      <c r="C23" s="17" t="s">
+      <c r="A23" s="45"/>
+      <c r="B23" s="45"/>
+      <c r="C23" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="D23" s="17">
+      <c r="D23" s="15">
         <v>3</v>
       </c>
-      <c r="E23" s="18">
+      <c r="E23" s="16">
         <f>SUM(D21:D23)</f>
         <v>6</v>
       </c>
-      <c r="F23" s="59"/>
-      <c r="G23" s="60"/>
-      <c r="H23" s="61"/>
+      <c r="F23" s="47"/>
+      <c r="G23" s="48"/>
+      <c r="H23" s="42"/>
     </row>
     <row r="24" ht="28.5">
-      <c r="A24" s="46">
+      <c r="A24" s="43">
         <v>46281</v>
       </c>
-      <c r="B24" s="46" t="s">
+      <c r="B24" s="43" t="s">
         <v>39</v>
       </c>
-      <c r="C24" s="28" t="s">
+      <c r="C24" s="25" t="s">
         <v>40</v>
       </c>
-      <c r="D24" s="28">
+      <c r="D24" s="25">
         <v>1</v>
       </c>
-      <c r="E24" s="29"/>
-      <c r="F24" s="62" t="s">
+      <c r="E24" s="26"/>
+      <c r="F24" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="G24" s="63">
-        <v>6</v>
-      </c>
-      <c r="H24" s="48"/>
+      <c r="G24" s="28">
+        <v>6</v>
+      </c>
+      <c r="H24" s="29"/>
     </row>
     <row r="25" ht="28.5">
-      <c r="A25" s="46"/>
-      <c r="B25" s="46"/>
-      <c r="C25" s="28" t="s">
+      <c r="A25" s="43"/>
+      <c r="B25" s="43"/>
+      <c r="C25" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="D25" s="28">
-        <v>2</v>
-      </c>
-      <c r="E25" s="34"/>
-      <c r="F25" s="35"/>
-      <c r="G25" s="36"/>
-      <c r="H25" s="50"/>
+      <c r="D25" s="25">
+        <v>2</v>
+      </c>
+      <c r="E25" s="31"/>
+      <c r="F25" s="32"/>
+      <c r="G25" s="33"/>
+      <c r="H25" s="34"/>
     </row>
     <row r="26" ht="28.5">
-      <c r="A26" s="46"/>
-      <c r="B26" s="46"/>
-      <c r="C26" s="28" t="s">
+      <c r="A26" s="43"/>
+      <c r="B26" s="43"/>
+      <c r="C26" s="25" t="s">
         <v>42</v>
       </c>
-      <c r="D26" s="28">
+      <c r="D26" s="25">
         <v>3</v>
       </c>
-      <c r="E26" s="34">
+      <c r="E26" s="31">
         <f>SUM(D24:D26)</f>
         <v>6</v>
       </c>
-      <c r="F26" s="64"/>
-      <c r="G26" s="51"/>
-      <c r="H26" s="52"/>
+      <c r="F26" s="49"/>
+      <c r="G26" s="44"/>
+      <c r="H26" s="37"/>
     </row>
     <row r="27" ht="28.5">
-      <c r="A27" s="15">
+      <c r="A27" s="14">
         <v>46282</v>
       </c>
-      <c r="B27" s="15" t="s">
+      <c r="B27" s="14" t="s">
         <v>43</v>
       </c>
-      <c r="C27" s="17" t="s">
+      <c r="C27" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="D27" s="17">
-        <v>2</v>
-      </c>
-      <c r="E27" s="18"/>
-      <c r="F27" s="65" t="s">
+      <c r="D27" s="15">
+        <v>2</v>
+      </c>
+      <c r="E27" s="16"/>
+      <c r="F27" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="G27" s="55">
-        <v>6</v>
-      </c>
-      <c r="H27" s="66"/>
+      <c r="G27" s="18">
+        <v>6</v>
+      </c>
+      <c r="H27" s="50"/>
     </row>
     <row r="28" ht="28.5">
-      <c r="A28" s="22"/>
-      <c r="B28" s="22"/>
-      <c r="C28" s="17" t="s">
+      <c r="A28" s="20"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="D28" s="17">
-        <v>2</v>
-      </c>
-      <c r="E28" s="18"/>
-      <c r="F28" s="67"/>
-      <c r="G28" s="24"/>
-      <c r="H28" s="21"/>
+      <c r="D28" s="15">
+        <v>2</v>
+      </c>
+      <c r="E28" s="16"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="22"/>
+      <c r="H28" s="19"/>
     </row>
     <row r="29" ht="28.5">
-      <c r="A29" s="25"/>
-      <c r="B29" s="25"/>
-      <c r="C29" s="68" t="s">
+      <c r="A29" s="23"/>
+      <c r="B29" s="23"/>
+      <c r="C29" s="51" t="s">
         <v>46</v>
       </c>
-      <c r="D29" s="17">
-        <v>2</v>
-      </c>
-      <c r="E29" s="18">
+      <c r="D29" s="15">
+        <v>2</v>
+      </c>
+      <c r="E29" s="16">
         <f>SUM(D27:D29)</f>
         <v>6</v>
       </c>
-      <c r="F29" s="69"/>
-      <c r="G29" s="44"/>
-      <c r="H29" s="70"/>
+      <c r="F29" s="52"/>
+      <c r="G29" s="41"/>
+      <c r="H29" s="53"/>
     </row>
     <row r="30" ht="28.5">
-      <c r="A30" s="46">
+      <c r="A30" s="43">
         <v>46283</v>
       </c>
-      <c r="B30" s="46" t="s">
+      <c r="B30" s="43" t="s">
         <v>47</v>
       </c>
-      <c r="C30" s="28" t="s">
+      <c r="C30" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="D30" s="28">
-        <v>2</v>
-      </c>
-      <c r="E30" s="29"/>
-      <c r="F30" s="71" t="s">
+      <c r="D30" s="25">
+        <v>2</v>
+      </c>
+      <c r="E30" s="26"/>
+      <c r="F30" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="G30" s="36">
-        <v>6</v>
-      </c>
-      <c r="H30" s="48"/>
+      <c r="G30" s="33">
+        <v>6</v>
+      </c>
+      <c r="H30" s="29"/>
     </row>
     <row r="31" ht="28.5">
-      <c r="A31" s="46"/>
-      <c r="B31" s="46"/>
-      <c r="C31" s="28" t="s">
+      <c r="A31" s="43"/>
+      <c r="B31" s="43"/>
+      <c r="C31" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="D31" s="28">
-        <v>2</v>
-      </c>
-      <c r="E31" s="34"/>
-      <c r="F31" s="72"/>
-      <c r="G31" s="36"/>
-      <c r="H31" s="50"/>
+      <c r="D31" s="25">
+        <v>2</v>
+      </c>
+      <c r="E31" s="31"/>
+      <c r="F31" s="32"/>
+      <c r="G31" s="33"/>
+      <c r="H31" s="34"/>
     </row>
     <row r="32" ht="32.25" customHeight="1">
-      <c r="A32" s="46"/>
-      <c r="B32" s="46"/>
-      <c r="C32" s="73" t="s">
+      <c r="A32" s="43"/>
+      <c r="B32" s="43"/>
+      <c r="C32" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D32" s="28">
-        <v>2</v>
-      </c>
-      <c r="E32" s="34">
+      <c r="D32" s="25">
+        <v>2</v>
+      </c>
+      <c r="E32" s="31">
         <f>SUM(D30:D32)</f>
         <v>6</v>
       </c>
-      <c r="F32" s="39"/>
-      <c r="G32" s="51"/>
-      <c r="H32" s="52"/>
+      <c r="F32" s="36"/>
+      <c r="G32" s="44"/>
+      <c r="H32" s="37"/>
     </row>
     <row r="33" ht="28.5">
-      <c r="A33" s="53">
+      <c r="A33" s="45">
         <v>46286</v>
       </c>
-      <c r="B33" s="53" t="s">
+      <c r="B33" s="45" t="s">
         <v>51</v>
       </c>
-      <c r="C33" s="17" t="s">
+      <c r="C33" s="15" t="s">
         <v>52</v>
       </c>
-      <c r="D33" s="17">
+      <c r="D33" s="15">
         <v>1</v>
       </c>
-      <c r="E33" s="18"/>
-      <c r="F33" s="54" t="s">
+      <c r="E33" s="16"/>
+      <c r="F33" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="G33" s="55">
-        <v>6</v>
-      </c>
-      <c r="H33" s="56"/>
+      <c r="G33" s="18">
+        <v>6</v>
+      </c>
+      <c r="H33" s="39"/>
     </row>
     <row r="34" ht="28.5">
-      <c r="A34" s="53"/>
-      <c r="B34" s="53"/>
-      <c r="C34" s="17" t="s">
+      <c r="A34" s="45"/>
+      <c r="B34" s="45"/>
+      <c r="C34" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="D34" s="17">
-        <v>2</v>
-      </c>
-      <c r="E34" s="18"/>
-      <c r="F34" s="57"/>
-      <c r="G34" s="24"/>
-      <c r="H34" s="58"/>
+      <c r="D34" s="15">
+        <v>2</v>
+      </c>
+      <c r="E34" s="16"/>
+      <c r="F34" s="38"/>
+      <c r="G34" s="22"/>
+      <c r="H34" s="40"/>
     </row>
     <row r="35" ht="28.5">
-      <c r="A35" s="53"/>
-      <c r="B35" s="53"/>
-      <c r="C35" s="17" t="s">
+      <c r="A35" s="45"/>
+      <c r="B35" s="45"/>
+      <c r="C35" s="15" t="s">
         <v>54</v>
       </c>
-      <c r="D35" s="17">
+      <c r="D35" s="15">
         <v>3</v>
       </c>
-      <c r="E35" s="18">
+      <c r="E35" s="16">
         <f>SUM(D33:D35)</f>
         <v>6</v>
       </c>
-      <c r="F35" s="74"/>
-      <c r="G35" s="60"/>
-      <c r="H35" s="61"/>
+      <c r="F35" s="54"/>
+      <c r="G35" s="48"/>
+      <c r="H35" s="42"/>
     </row>
     <row r="36" ht="28.5">
-      <c r="A36" s="26">
+      <c r="A36" s="24">
         <v>46287</v>
       </c>
-      <c r="B36" s="26" t="s">
+      <c r="B36" s="24" t="s">
         <v>55</v>
       </c>
-      <c r="C36" s="28" t="s">
+      <c r="C36" s="25" t="s">
         <v>56</v>
       </c>
-      <c r="D36" s="28">
-        <v>2</v>
-      </c>
-      <c r="E36" s="29"/>
-      <c r="F36" s="71" t="s">
+      <c r="D36" s="25">
+        <v>2</v>
+      </c>
+      <c r="E36" s="26"/>
+      <c r="F36" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="G36" s="63">
-        <v>6</v>
-      </c>
-      <c r="H36" s="48"/>
+      <c r="G36" s="28">
+        <v>6</v>
+      </c>
+      <c r="H36" s="29"/>
     </row>
     <row r="37" ht="28.5">
-      <c r="A37" s="46"/>
-      <c r="B37" s="33"/>
-      <c r="C37" s="28" t="s">
+      <c r="A37" s="43"/>
+      <c r="B37" s="30"/>
+      <c r="C37" s="25" t="s">
         <v>57</v>
       </c>
-      <c r="D37" s="28">
-        <v>2</v>
-      </c>
-      <c r="E37" s="34"/>
-      <c r="F37" s="72"/>
-      <c r="G37" s="36"/>
-      <c r="H37" s="50"/>
+      <c r="D37" s="25">
+        <v>2</v>
+      </c>
+      <c r="E37" s="31"/>
+      <c r="F37" s="32"/>
+      <c r="G37" s="33"/>
+      <c r="H37" s="34"/>
     </row>
     <row r="38" ht="28.5">
-      <c r="A38" s="38"/>
-      <c r="B38" s="38"/>
-      <c r="C38" s="28" t="s">
+      <c r="A38" s="35"/>
+      <c r="B38" s="35"/>
+      <c r="C38" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="D38" s="28">
-        <v>2</v>
-      </c>
-      <c r="E38" s="34">
+      <c r="D38" s="25">
+        <v>2</v>
+      </c>
+      <c r="E38" s="31">
         <f>SUM(D36:D38)</f>
         <v>6</v>
       </c>
-      <c r="F38" s="39"/>
-      <c r="G38" s="51"/>
-      <c r="H38" s="52"/>
+      <c r="F38" s="36"/>
+      <c r="G38" s="44"/>
+      <c r="H38" s="37"/>
     </row>
     <row r="39" ht="28.5">
-      <c r="A39" s="15">
+      <c r="A39" s="14">
         <v>46288</v>
       </c>
-      <c r="B39" s="53" t="s">
+      <c r="B39" s="45" t="s">
         <v>59</v>
       </c>
-      <c r="C39" s="17" t="s">
+      <c r="C39" s="15" t="s">
         <v>60</v>
       </c>
-      <c r="D39" s="17">
+      <c r="D39" s="15">
         <v>1</v>
       </c>
-      <c r="E39" s="18"/>
-      <c r="F39" s="54" t="s">
+      <c r="E39" s="16"/>
+      <c r="F39" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="G39" s="55">
-        <v>6</v>
-      </c>
-      <c r="H39" s="56"/>
+      <c r="G39" s="18">
+        <v>6</v>
+      </c>
+      <c r="H39" s="39"/>
     </row>
     <row r="40" ht="28.5">
-      <c r="A40" s="53"/>
-      <c r="B40" s="53"/>
-      <c r="C40" s="17" t="s">
+      <c r="A40" s="45"/>
+      <c r="B40" s="45"/>
+      <c r="C40" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="D40" s="17">
+      <c r="D40" s="15">
         <v>3</v>
       </c>
-      <c r="E40" s="18"/>
-      <c r="F40" s="57"/>
-      <c r="G40" s="24"/>
-      <c r="H40" s="58"/>
+      <c r="E40" s="16"/>
+      <c r="F40" s="38"/>
+      <c r="G40" s="22"/>
+      <c r="H40" s="40"/>
     </row>
     <row r="41" ht="28.5">
-      <c r="A41" s="25"/>
-      <c r="B41" s="53"/>
-      <c r="C41" s="17" t="s">
+      <c r="A41" s="23"/>
+      <c r="B41" s="45"/>
+      <c r="C41" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="D41" s="17">
-        <v>2</v>
-      </c>
-      <c r="E41" s="18">
+      <c r="D41" s="15">
+        <v>2</v>
+      </c>
+      <c r="E41" s="16">
         <f>SUM(D39:D41)</f>
         <v>6</v>
       </c>
-      <c r="F41" s="41"/>
-      <c r="G41" s="44"/>
-      <c r="H41" s="61"/>
+      <c r="F41" s="38"/>
+      <c r="G41" s="41"/>
+      <c r="H41" s="42"/>
     </row>
     <row r="42" ht="28.5">
-      <c r="A42" s="26">
+      <c r="A42" s="24">
         <v>46289</v>
       </c>
-      <c r="B42" s="46" t="s">
+      <c r="B42" s="43" t="s">
         <v>63</v>
       </c>
-      <c r="C42" s="28" t="s">
+      <c r="C42" s="25" t="s">
         <v>64</v>
       </c>
-      <c r="D42" s="28">
-        <v>2</v>
-      </c>
-      <c r="E42" s="29"/>
-      <c r="F42" s="47" t="s">
+      <c r="D42" s="25">
+        <v>2</v>
+      </c>
+      <c r="E42" s="26"/>
+      <c r="F42" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="G42" s="75">
-        <v>6</v>
-      </c>
-      <c r="H42" s="48"/>
+      <c r="G42" s="33">
+        <v>6</v>
+      </c>
+      <c r="H42" s="29"/>
     </row>
     <row r="43" ht="28.5">
-      <c r="A43" s="46"/>
-      <c r="B43" s="46"/>
-      <c r="C43" s="28" t="s">
+      <c r="A43" s="43"/>
+      <c r="B43" s="43"/>
+      <c r="C43" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="D43" s="28">
-        <v>2</v>
-      </c>
-      <c r="E43" s="34"/>
-      <c r="F43" s="49"/>
-      <c r="G43" s="75"/>
-      <c r="H43" s="50"/>
+      <c r="D43" s="25">
+        <v>2</v>
+      </c>
+      <c r="E43" s="31"/>
+      <c r="F43" s="32"/>
+      <c r="G43" s="33"/>
+      <c r="H43" s="34"/>
     </row>
     <row r="44">
-      <c r="A44" s="38"/>
-      <c r="B44" s="46"/>
-      <c r="C44" s="28" t="s">
+      <c r="A44" s="35"/>
+      <c r="B44" s="43"/>
+      <c r="C44" s="25" t="s">
         <v>66</v>
       </c>
-      <c r="D44" s="28">
-        <v>2</v>
-      </c>
-      <c r="E44" s="34">
+      <c r="D44" s="25">
+        <v>2</v>
+      </c>
+      <c r="E44" s="31">
         <f>SUM(D42:D44)</f>
         <v>6</v>
       </c>
-      <c r="F44" s="39"/>
-      <c r="G44" s="76"/>
-      <c r="H44" s="52"/>
+      <c r="F44" s="36"/>
+      <c r="G44" s="44"/>
+      <c r="H44" s="37"/>
     </row>
     <row r="45" ht="28.5">
-      <c r="A45" s="15">
+      <c r="A45" s="14">
         <v>46290</v>
       </c>
-      <c r="B45" s="77" t="s">
+      <c r="B45" s="45" t="s">
         <v>67</v>
       </c>
-      <c r="C45" s="16" t="s">
+      <c r="C45" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="D45" s="17">
-        <v>2</v>
-      </c>
-      <c r="E45" s="18"/>
-      <c r="F45" s="54" t="s">
+      <c r="D45" s="15">
+        <v>2</v>
+      </c>
+      <c r="E45" s="16"/>
+      <c r="F45" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="G45" s="78">
-        <v>6</v>
-      </c>
-      <c r="H45" s="66"/>
+      <c r="G45" s="18">
+        <v>6</v>
+      </c>
+      <c r="H45" s="50"/>
     </row>
     <row r="46" ht="28.5">
-      <c r="A46" s="53"/>
-      <c r="B46" s="53"/>
-      <c r="C46" s="16" t="s">
+      <c r="A46" s="45"/>
+      <c r="B46" s="45"/>
+      <c r="C46" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="D46" s="17">
-        <v>2</v>
-      </c>
-      <c r="E46" s="18"/>
-      <c r="F46" s="57"/>
-      <c r="G46" s="79"/>
-      <c r="H46" s="21"/>
+      <c r="D46" s="15">
+        <v>2</v>
+      </c>
+      <c r="E46" s="16"/>
+      <c r="F46" s="38"/>
+      <c r="G46" s="22"/>
+      <c r="H46" s="19"/>
     </row>
     <row r="47" ht="28.5">
-      <c r="A47" s="25"/>
-      <c r="B47" s="53"/>
-      <c r="C47" s="16" t="s">
+      <c r="A47" s="23"/>
+      <c r="B47" s="45"/>
+      <c r="C47" s="15" t="s">
         <v>70</v>
       </c>
-      <c r="D47" s="17">
-        <v>2</v>
-      </c>
-      <c r="E47" s="18">
+      <c r="D47" s="15">
+        <v>2</v>
+      </c>
+      <c r="E47" s="16">
         <f>SUM(D45:D47)</f>
         <v>6</v>
       </c>
-      <c r="F47" s="74"/>
-      <c r="G47" s="80"/>
-      <c r="H47" s="70"/>
+      <c r="F47" s="54"/>
+      <c r="G47" s="48"/>
+      <c r="H47" s="53"/>
     </row>
     <row r="48" ht="28.5">
-      <c r="A48" s="46">
+      <c r="A48" s="43">
         <v>46293</v>
       </c>
-      <c r="B48" s="46" t="s">
+      <c r="B48" s="43" t="s">
         <v>71</v>
       </c>
-      <c r="C48" s="28" t="s">
+      <c r="C48" s="25" t="s">
         <v>72</v>
       </c>
-      <c r="D48" s="28">
-        <v>2</v>
-      </c>
-      <c r="E48" s="29"/>
-      <c r="F48" s="71" t="s">
+      <c r="D48" s="25">
+        <v>2</v>
+      </c>
+      <c r="E48" s="26"/>
+      <c r="F48" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="G48" s="81">
-        <v>6</v>
-      </c>
-      <c r="H48" s="48"/>
+      <c r="G48" s="28">
+        <v>6</v>
+      </c>
+      <c r="H48" s="29"/>
     </row>
     <row r="49" ht="28.5">
-      <c r="A49" s="46"/>
-      <c r="B49" s="46"/>
-      <c r="C49" s="28" t="s">
+      <c r="A49" s="43"/>
+      <c r="B49" s="43"/>
+      <c r="C49" s="25" t="s">
         <v>73</v>
       </c>
-      <c r="D49" s="28">
-        <v>2</v>
-      </c>
-      <c r="E49" s="34"/>
-      <c r="F49" s="72"/>
-      <c r="G49" s="75"/>
-      <c r="H49" s="50"/>
+      <c r="D49" s="25">
+        <v>2</v>
+      </c>
+      <c r="E49" s="31"/>
+      <c r="F49" s="32"/>
+      <c r="G49" s="33"/>
+      <c r="H49" s="34"/>
     </row>
     <row r="50" ht="28.5">
-      <c r="A50" s="46"/>
-      <c r="B50" s="46"/>
-      <c r="C50" s="28" t="s">
+      <c r="A50" s="43"/>
+      <c r="B50" s="43"/>
+      <c r="C50" s="25" t="s">
         <v>74</v>
       </c>
-      <c r="D50" s="28">
-        <v>2</v>
-      </c>
-      <c r="E50" s="34">
+      <c r="D50" s="25">
+        <v>2</v>
+      </c>
+      <c r="E50" s="31">
         <f>SUM(D48:D50)</f>
         <v>6</v>
       </c>
-      <c r="F50" s="39"/>
-      <c r="G50" s="76"/>
-      <c r="H50" s="52"/>
+      <c r="F50" s="36"/>
+      <c r="G50" s="44"/>
+      <c r="H50" s="37"/>
     </row>
     <row r="51" ht="28.5">
-      <c r="A51" s="53">
+      <c r="A51" s="45">
         <v>46294</v>
       </c>
-      <c r="B51" s="53" t="s">
+      <c r="B51" s="45" t="s">
         <v>75</v>
       </c>
-      <c r="C51" s="17" t="s">
+      <c r="C51" s="15" t="s">
         <v>76</v>
       </c>
-      <c r="D51" s="17">
-        <v>2</v>
-      </c>
-      <c r="E51" s="18"/>
-      <c r="F51" s="54" t="s">
+      <c r="D51" s="15">
+        <v>2</v>
+      </c>
+      <c r="E51" s="16"/>
+      <c r="F51" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="G51" s="78">
-        <v>6</v>
-      </c>
-      <c r="H51" s="56"/>
+      <c r="G51" s="18">
+        <v>6</v>
+      </c>
+      <c r="H51" s="39"/>
     </row>
     <row r="52">
-      <c r="A52" s="53"/>
-      <c r="B52" s="53"/>
-      <c r="C52" s="17" t="s">
+      <c r="A52" s="45"/>
+      <c r="B52" s="45"/>
+      <c r="C52" s="15" t="s">
         <v>77</v>
       </c>
-      <c r="D52" s="17">
-        <v>2</v>
-      </c>
-      <c r="E52" s="18"/>
-      <c r="F52" s="57"/>
-      <c r="G52" s="79"/>
-      <c r="H52" s="58"/>
+      <c r="D52" s="15">
+        <v>2</v>
+      </c>
+      <c r="E52" s="16"/>
+      <c r="F52" s="38"/>
+      <c r="G52" s="22"/>
+      <c r="H52" s="40"/>
     </row>
     <row r="53" ht="28.5">
-      <c r="A53" s="53"/>
-      <c r="B53" s="53"/>
-      <c r="C53" s="17" t="s">
+      <c r="A53" s="45"/>
+      <c r="B53" s="45"/>
+      <c r="C53" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="D53" s="17">
-        <v>2</v>
-      </c>
-      <c r="E53" s="18">
+      <c r="D53" s="15">
+        <v>2</v>
+      </c>
+      <c r="E53" s="16">
         <f>SUM(D51:D53)</f>
         <v>6</v>
       </c>
-      <c r="F53" s="59"/>
-      <c r="G53" s="44"/>
-      <c r="H53" s="61"/>
+      <c r="F53" s="47"/>
+      <c r="G53" s="41"/>
+      <c r="H53" s="42"/>
     </row>
     <row r="54" ht="28.5">
-      <c r="A54" s="46">
+      <c r="A54" s="43">
         <v>46295</v>
       </c>
-      <c r="B54" s="46" t="s">
+      <c r="B54" s="43" t="s">
         <v>79</v>
       </c>
-      <c r="C54" s="28" t="s">
+      <c r="C54" s="25" t="s">
         <v>80</v>
       </c>
-      <c r="D54" s="28">
-        <v>2</v>
-      </c>
-      <c r="E54" s="29"/>
-      <c r="F54" s="72" t="s">
+      <c r="D54" s="25">
+        <v>2</v>
+      </c>
+      <c r="E54" s="26"/>
+      <c r="F54" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="G54" s="82">
-        <v>6</v>
-      </c>
-      <c r="H54" s="48"/>
+      <c r="G54" s="33">
+        <v>6</v>
+      </c>
+      <c r="H54" s="29"/>
     </row>
     <row r="55" ht="28.5">
-      <c r="A55" s="46"/>
-      <c r="B55" s="46"/>
-      <c r="C55" s="28" t="s">
+      <c r="A55" s="43"/>
+      <c r="B55" s="43"/>
+      <c r="C55" s="25" t="s">
         <v>81</v>
       </c>
-      <c r="D55" s="28">
-        <v>2</v>
-      </c>
-      <c r="E55" s="34"/>
-      <c r="F55" s="72"/>
-      <c r="G55" s="83"/>
-      <c r="H55" s="50"/>
+      <c r="D55" s="25">
+        <v>2</v>
+      </c>
+      <c r="E55" s="31"/>
+      <c r="F55" s="32"/>
+      <c r="G55" s="33"/>
+      <c r="H55" s="34"/>
     </row>
     <row r="56" ht="28.5">
-      <c r="A56" s="46"/>
-      <c r="B56" s="46"/>
-      <c r="C56" s="28" t="s">
+      <c r="A56" s="43"/>
+      <c r="B56" s="43"/>
+      <c r="C56" s="55" t="s">
         <v>82</v>
       </c>
-      <c r="D56" s="28">
-        <v>2</v>
-      </c>
-      <c r="E56" s="34">
+      <c r="D56" s="25">
+        <v>2</v>
+      </c>
+      <c r="E56" s="31">
         <f>SUM(D54:D56)</f>
         <v>6</v>
       </c>
-      <c r="F56" s="84"/>
-      <c r="G56" s="85"/>
-      <c r="H56" s="52"/>
+      <c r="F56" s="49"/>
+      <c r="G56" s="44"/>
+      <c r="H56" s="37"/>
     </row>
     <row r="57" ht="28.5">
-      <c r="A57" s="53">
+      <c r="A57" s="45">
         <v>46296</v>
       </c>
-      <c r="B57" s="53" t="s">
+      <c r="B57" s="45" t="s">
         <v>83</v>
       </c>
-      <c r="C57" s="17" t="s">
+      <c r="C57" s="15" t="s">
         <v>84</v>
       </c>
-      <c r="D57" s="17">
-        <v>2</v>
-      </c>
-      <c r="E57" s="18"/>
-      <c r="F57" s="65" t="s">
+      <c r="D57" s="15">
+        <v>2</v>
+      </c>
+      <c r="E57" s="16"/>
+      <c r="F57" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="G57" s="78">
-        <v>6</v>
-      </c>
-      <c r="H57" s="56"/>
+      <c r="G57" s="18">
+        <v>6</v>
+      </c>
+      <c r="H57" s="39"/>
     </row>
     <row r="58" ht="28.5">
-      <c r="A58" s="53"/>
-      <c r="B58" s="53"/>
-      <c r="C58" s="17" t="s">
+      <c r="A58" s="45"/>
+      <c r="B58" s="45"/>
+      <c r="C58" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="D58" s="17">
-        <v>2</v>
-      </c>
-      <c r="E58" s="18"/>
-      <c r="F58" s="67"/>
-      <c r="G58" s="79"/>
-      <c r="H58" s="58"/>
+      <c r="D58" s="15">
+        <v>2</v>
+      </c>
+      <c r="E58" s="16"/>
+      <c r="F58" s="21"/>
+      <c r="G58" s="22"/>
+      <c r="H58" s="40"/>
     </row>
     <row r="59" ht="28.5">
-      <c r="A59" s="53"/>
-      <c r="B59" s="53"/>
-      <c r="C59" s="17" t="s">
+      <c r="A59" s="45"/>
+      <c r="B59" s="45"/>
+      <c r="C59" s="15" t="s">
         <v>86</v>
       </c>
-      <c r="D59" s="17">
-        <v>2</v>
-      </c>
-      <c r="E59" s="18">
+      <c r="D59" s="15">
+        <v>2</v>
+      </c>
+      <c r="E59" s="16">
         <f>SUM(D57:D59)</f>
         <v>6</v>
       </c>
-      <c r="F59" s="69"/>
-      <c r="G59" s="80"/>
-      <c r="H59" s="61"/>
+      <c r="F59" s="52"/>
+      <c r="G59" s="48"/>
+      <c r="H59" s="42"/>
     </row>
     <row r="60" ht="28.5">
-      <c r="A60" s="46">
+      <c r="A60" s="43">
         <v>46297</v>
       </c>
-      <c r="B60" s="46" t="s">
+      <c r="B60" s="43" t="s">
         <v>87</v>
       </c>
-      <c r="C60" s="28" t="s">
+      <c r="C60" s="25" t="s">
         <v>88</v>
       </c>
-      <c r="D60" s="28">
-        <v>2</v>
-      </c>
-      <c r="E60" s="29"/>
-      <c r="F60" s="71" t="s">
+      <c r="D60" s="25">
+        <v>2</v>
+      </c>
+      <c r="E60" s="26"/>
+      <c r="F60" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="G60" s="81">
-        <v>6</v>
-      </c>
-      <c r="H60" s="48"/>
+      <c r="G60" s="28">
+        <v>6</v>
+      </c>
+      <c r="H60" s="29"/>
     </row>
     <row r="61" ht="28.5">
-      <c r="A61" s="46"/>
-      <c r="B61" s="46"/>
-      <c r="C61" s="28" t="s">
+      <c r="A61" s="43"/>
+      <c r="B61" s="43"/>
+      <c r="C61" s="25" t="s">
         <v>89</v>
       </c>
-      <c r="D61" s="28">
-        <v>2</v>
-      </c>
-      <c r="E61" s="34"/>
-      <c r="F61" s="72"/>
-      <c r="G61" s="75"/>
-      <c r="H61" s="50"/>
+      <c r="D61" s="25">
+        <v>2</v>
+      </c>
+      <c r="E61" s="31"/>
+      <c r="F61" s="32"/>
+      <c r="G61" s="33"/>
+      <c r="H61" s="34"/>
     </row>
     <row r="62" ht="28.5">
-      <c r="A62" s="46"/>
-      <c r="B62" s="46"/>
-      <c r="C62" s="28" t="s">
+      <c r="A62" s="43"/>
+      <c r="B62" s="43"/>
+      <c r="C62" s="55" t="s">
         <v>90</v>
       </c>
-      <c r="D62" s="28">
-        <v>2</v>
-      </c>
-      <c r="E62" s="34">
+      <c r="D62" s="25">
+        <v>2</v>
+      </c>
+      <c r="E62" s="31">
         <f>SUM(D60:D62)</f>
         <v>6</v>
       </c>
-      <c r="F62" s="39"/>
-      <c r="G62" s="76"/>
-      <c r="H62" s="52"/>
+      <c r="F62" s="36"/>
+      <c r="G62" s="44"/>
+      <c r="H62" s="37"/>
     </row>
     <row r="63" ht="28.5">
-      <c r="A63" s="53">
+      <c r="A63" s="45">
         <v>46300</v>
       </c>
-      <c r="B63" s="53" t="s">
+      <c r="B63" s="45" t="s">
         <v>91</v>
       </c>
-      <c r="C63" s="17" t="s">
+      <c r="C63" s="15" t="s">
         <v>92</v>
       </c>
-      <c r="D63" s="17">
-        <v>2</v>
-      </c>
-      <c r="E63" s="18"/>
-      <c r="F63" s="54" t="s">
+      <c r="D63" s="15">
+        <v>2</v>
+      </c>
+      <c r="E63" s="16"/>
+      <c r="F63" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="G63" s="78">
-        <v>6</v>
-      </c>
-      <c r="H63" s="66"/>
+      <c r="G63" s="18">
+        <v>6</v>
+      </c>
+      <c r="H63" s="50"/>
     </row>
     <row r="64" ht="28.5">
-      <c r="A64" s="53"/>
-      <c r="B64" s="53"/>
-      <c r="C64" s="17" t="s">
+      <c r="A64" s="45"/>
+      <c r="B64" s="45"/>
+      <c r="C64" s="15" t="s">
         <v>93</v>
       </c>
-      <c r="D64" s="17">
-        <v>2</v>
-      </c>
-      <c r="E64" s="18"/>
-      <c r="F64" s="57"/>
-      <c r="G64" s="79"/>
-      <c r="H64" s="21"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="53"/>
-      <c r="B65" s="53"/>
-      <c r="C65" s="17" t="s">
+      <c r="D64" s="15">
+        <v>2</v>
+      </c>
+      <c r="E64" s="16"/>
+      <c r="F64" s="38"/>
+      <c r="G64" s="22"/>
+      <c r="H64" s="19"/>
+    </row>
+    <row r="65" ht="28.5">
+      <c r="A65" s="45"/>
+      <c r="B65" s="45"/>
+      <c r="C65" s="56" t="s">
         <v>94</v>
       </c>
-      <c r="D65" s="17">
-        <v>2</v>
-      </c>
-      <c r="E65" s="18">
+      <c r="D65" s="15">
+        <v>2</v>
+      </c>
+      <c r="E65" s="16">
         <f>SUM(D63:D65)</f>
         <v>6</v>
       </c>
-      <c r="F65" s="74"/>
-      <c r="G65" s="44"/>
-      <c r="H65" s="70"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="46">
+      <c r="F65" s="54"/>
+      <c r="G65" s="41"/>
+      <c r="H65" s="53"/>
+    </row>
+    <row r="66" ht="28.5">
+      <c r="A66" s="43">
         <v>46301</v>
       </c>
-      <c r="B66" s="86" t="s">
+      <c r="B66" s="57" t="s">
         <v>95</v>
       </c>
-      <c r="C66" s="27" t="s">
+      <c r="C66" s="25" t="s">
         <v>96</v>
       </c>
-      <c r="D66" s="28">
+      <c r="D66" s="25">
         <v>1</v>
       </c>
-      <c r="E66" s="29"/>
-      <c r="F66" s="71" t="s">
+      <c r="E66" s="26"/>
+      <c r="F66" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="G66" s="75">
-        <v>6</v>
-      </c>
-      <c r="H66" s="48"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="46"/>
-      <c r="B67" s="86"/>
-      <c r="C67" s="27" t="s">
+      <c r="G66" s="33">
+        <v>6</v>
+      </c>
+      <c r="H66" s="29"/>
+    </row>
+    <row r="67" ht="28.5">
+      <c r="A67" s="43"/>
+      <c r="B67" s="57"/>
+      <c r="C67" s="25" t="s">
         <v>97</v>
       </c>
-      <c r="D67" s="28">
+      <c r="D67" s="25">
         <v>3</v>
       </c>
-      <c r="E67" s="34"/>
-      <c r="F67" s="72"/>
-      <c r="G67" s="75"/>
-      <c r="H67" s="50"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="46"/>
-      <c r="B68" s="86"/>
-      <c r="C68" s="27" t="s">
+      <c r="E67" s="31"/>
+      <c r="F67" s="32"/>
+      <c r="G67" s="33"/>
+      <c r="H67" s="34"/>
+    </row>
+    <row r="68" ht="28.5">
+      <c r="A68" s="43"/>
+      <c r="B68" s="57"/>
+      <c r="C68" s="25" t="s">
         <v>98</v>
       </c>
-      <c r="D68" s="28">
-        <v>2</v>
-      </c>
-      <c r="E68" s="34">
+      <c r="D68" s="25">
+        <v>2</v>
+      </c>
+      <c r="E68" s="31">
         <f>SUM(D66:D68)</f>
         <v>6</v>
       </c>
-      <c r="F68" s="39"/>
-      <c r="G68" s="76"/>
-      <c r="H68" s="52"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="53">
+      <c r="F68" s="36"/>
+      <c r="G68" s="44"/>
+      <c r="H68" s="37"/>
+    </row>
+    <row r="69" ht="28.5">
+      <c r="A69" s="45">
         <v>46302</v>
       </c>
-      <c r="B69" s="53" t="s">
+      <c r="B69" s="45" t="s">
         <v>99</v>
       </c>
-      <c r="C69" s="17" t="s">
+      <c r="C69" s="15" t="s">
         <v>100</v>
       </c>
-      <c r="D69" s="17">
-        <v>2</v>
-      </c>
-      <c r="E69" s="18"/>
-      <c r="F69" s="54" t="s">
+      <c r="D69" s="15">
+        <v>2</v>
+      </c>
+      <c r="E69" s="16"/>
+      <c r="F69" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="G69" s="78">
-        <v>6</v>
-      </c>
-      <c r="H69" s="56"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="53"/>
-      <c r="B70" s="53"/>
-      <c r="C70" s="17" t="s">
+      <c r="G69" s="18">
+        <v>6</v>
+      </c>
+      <c r="H69" s="39"/>
+    </row>
+    <row r="70" ht="28.5">
+      <c r="A70" s="45"/>
+      <c r="B70" s="45"/>
+      <c r="C70" s="15" t="s">
         <v>101</v>
       </c>
-      <c r="D70" s="17">
-        <v>2</v>
-      </c>
-      <c r="E70" s="18"/>
-      <c r="F70" s="57"/>
-      <c r="G70" s="79"/>
-      <c r="H70" s="58"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="53"/>
-      <c r="B71" s="53"/>
-      <c r="C71" s="17" t="s">
+      <c r="D70" s="15">
+        <v>2</v>
+      </c>
+      <c r="E70" s="16"/>
+      <c r="F70" s="38"/>
+      <c r="G70" s="22"/>
+      <c r="H70" s="40"/>
+    </row>
+    <row r="71" ht="28.5">
+      <c r="A71" s="45"/>
+      <c r="B71" s="45"/>
+      <c r="C71" s="15" t="s">
         <v>102</v>
       </c>
-      <c r="D71" s="17">
-        <v>2</v>
-      </c>
-      <c r="E71" s="18">
+      <c r="D71" s="15">
+        <v>2</v>
+      </c>
+      <c r="E71" s="16">
         <f>SUM(D69:D71)</f>
         <v>6</v>
       </c>
-      <c r="F71" s="41"/>
-      <c r="G71" s="80"/>
-      <c r="H71" s="61"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="46">
+      <c r="F71" s="38"/>
+      <c r="G71" s="48"/>
+      <c r="H71" s="42"/>
+    </row>
+    <row r="72" ht="28.5">
+      <c r="A72" s="43">
         <v>46303</v>
       </c>
-      <c r="B72" s="46" t="s">
+      <c r="B72" s="43" t="s">
         <v>103</v>
       </c>
-      <c r="C72" s="27" t="s">
+      <c r="C72" s="25" t="s">
         <v>104</v>
       </c>
-      <c r="D72" s="28">
+      <c r="D72" s="25">
         <v>1</v>
       </c>
-      <c r="E72" s="29"/>
-      <c r="F72" s="47" t="s">
+      <c r="E72" s="26"/>
+      <c r="F72" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="G72" s="81">
-        <v>6</v>
-      </c>
-      <c r="H72" s="48"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="46"/>
-      <c r="B73" s="46"/>
-      <c r="C73" s="27" t="s">
+      <c r="G72" s="28">
+        <v>6</v>
+      </c>
+      <c r="H72" s="29"/>
+    </row>
+    <row r="73" ht="28.5">
+      <c r="A73" s="43"/>
+      <c r="B73" s="43"/>
+      <c r="C73" s="55" t="s">
         <v>105</v>
       </c>
-      <c r="D73" s="28">
+      <c r="D73" s="25">
         <v>3</v>
       </c>
-      <c r="E73" s="34"/>
-      <c r="F73" s="49"/>
-      <c r="G73" s="75"/>
-      <c r="H73" s="50"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="46"/>
-      <c r="B74" s="46"/>
-      <c r="C74" s="27" t="s">
+      <c r="E73" s="31"/>
+      <c r="F73" s="32"/>
+      <c r="G73" s="33"/>
+      <c r="H73" s="34"/>
+    </row>
+    <row r="74" ht="28.5">
+      <c r="A74" s="43"/>
+      <c r="B74" s="43"/>
+      <c r="C74" s="55" t="s">
         <v>106</v>
       </c>
-      <c r="D74" s="28">
-        <v>2</v>
-      </c>
-      <c r="E74" s="34">
+      <c r="D74" s="25">
+        <v>2</v>
+      </c>
+      <c r="E74" s="31">
         <f>SUM(D72:D74)</f>
         <v>6</v>
       </c>
-      <c r="F74" s="39"/>
-      <c r="G74" s="76"/>
-      <c r="H74" s="52"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="87">
+      <c r="F74" s="36"/>
+      <c r="G74" s="44"/>
+      <c r="H74" s="37"/>
+    </row>
+    <row r="75" ht="28.5">
+      <c r="A75" s="58">
         <v>46307</v>
       </c>
-      <c r="B75" s="88" t="s">
+      <c r="B75" s="58" t="s">
         <v>107</v>
       </c>
-      <c r="C75" s="89" t="s">
+      <c r="C75" s="59" t="s">
         <v>108</v>
       </c>
-      <c r="D75" s="17">
-        <v>2</v>
-      </c>
-      <c r="E75" s="18"/>
-      <c r="F75" s="54" t="s">
+      <c r="D75" s="15">
+        <v>2</v>
+      </c>
+      <c r="E75" s="16"/>
+      <c r="F75" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="G75" s="78">
-        <v>6</v>
-      </c>
-      <c r="H75" s="56"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="87"/>
-      <c r="B76" s="87"/>
-      <c r="C76" s="89" t="s">
+      <c r="G75" s="18">
+        <v>6</v>
+      </c>
+      <c r="H75" s="39"/>
+    </row>
+    <row r="76" ht="28.5">
+      <c r="A76" s="58"/>
+      <c r="B76" s="58"/>
+      <c r="C76" s="59" t="s">
         <v>109</v>
       </c>
-      <c r="D76" s="17">
-        <v>2</v>
-      </c>
-      <c r="E76" s="18"/>
-      <c r="F76" s="57"/>
-      <c r="G76" s="79"/>
-      <c r="H76" s="58"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="87"/>
-      <c r="B77" s="87"/>
-      <c r="C77" s="89" t="s">
+      <c r="D76" s="15">
+        <v>2</v>
+      </c>
+      <c r="E76" s="16"/>
+      <c r="F76" s="38"/>
+      <c r="G76" s="22"/>
+      <c r="H76" s="40"/>
+    </row>
+    <row r="77" ht="28.5">
+      <c r="A77" s="58"/>
+      <c r="B77" s="58"/>
+      <c r="C77" s="59" t="s">
         <v>110</v>
       </c>
-      <c r="D77" s="17">
-        <v>2</v>
-      </c>
-      <c r="E77" s="18">
+      <c r="D77" s="15">
+        <v>2</v>
+      </c>
+      <c r="E77" s="16">
         <f>SUM(D75:D77)</f>
         <v>6</v>
       </c>
-      <c r="F77" s="74"/>
-      <c r="G77" s="44"/>
-      <c r="H77" s="61"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="46">
+      <c r="F77" s="54"/>
+      <c r="G77" s="41"/>
+      <c r="H77" s="42"/>
+    </row>
+    <row r="78" ht="28.5">
+      <c r="A78" s="43">
         <v>46308</v>
       </c>
-      <c r="B78" s="90" t="s">
+      <c r="B78" s="43" t="s">
         <v>111</v>
       </c>
-      <c r="C78" s="27" t="s">
+      <c r="C78" s="25" t="s">
         <v>112</v>
       </c>
-      <c r="D78" s="28">
-        <v>2</v>
-      </c>
-      <c r="E78" s="29"/>
-      <c r="F78" s="71" t="s">
+      <c r="D78" s="25">
+        <v>2</v>
+      </c>
+      <c r="E78" s="26"/>
+      <c r="F78" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="G78" s="82">
-        <v>6</v>
-      </c>
-      <c r="H78" s="48"/>
+      <c r="G78" s="33">
+        <v>6</v>
+      </c>
+      <c r="H78" s="29"/>
     </row>
     <row r="79" ht="43.5" customHeight="1">
-      <c r="A79" s="46"/>
-      <c r="B79" s="46"/>
-      <c r="C79" s="27" t="s">
+      <c r="A79" s="43"/>
+      <c r="B79" s="43"/>
+      <c r="C79" s="25" t="s">
         <v>113</v>
       </c>
-      <c r="D79" s="28">
+      <c r="D79" s="25">
         <v>3</v>
       </c>
-      <c r="E79" s="34"/>
-      <c r="F79" s="72"/>
-      <c r="G79" s="83"/>
-      <c r="H79" s="50"/>
+      <c r="E79" s="31"/>
+      <c r="F79" s="32"/>
+      <c r="G79" s="33"/>
+      <c r="H79" s="34"/>
     </row>
     <row r="80" ht="38.25" customHeight="1">
-      <c r="A80" s="46"/>
-      <c r="B80" s="46"/>
-      <c r="C80" s="28" t="s">
+      <c r="A80" s="43"/>
+      <c r="B80" s="43"/>
+      <c r="C80" s="25" t="s">
         <v>114</v>
       </c>
-      <c r="D80" s="28">
+      <c r="D80" s="25">
         <v>1</v>
       </c>
-      <c r="E80" s="34">
+      <c r="E80" s="31">
         <f>SUM(D78:D80)</f>
         <v>6</v>
       </c>
-      <c r="F80" s="39"/>
-      <c r="G80" s="85"/>
-      <c r="H80" s="52"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="87">
+      <c r="F80" s="36"/>
+      <c r="G80" s="44"/>
+      <c r="H80" s="37"/>
+    </row>
+    <row r="81" ht="28.5">
+      <c r="A81" s="58">
         <v>46309</v>
       </c>
-      <c r="B81" s="91" t="s">
+      <c r="B81" s="60" t="s">
         <v>115</v>
       </c>
-      <c r="C81" s="89" t="s">
+      <c r="C81" s="59" t="s">
         <v>116</v>
       </c>
-      <c r="D81" s="17">
-        <v>2</v>
-      </c>
-      <c r="E81" s="18"/>
-      <c r="F81" s="54" t="s">
+      <c r="D81" s="15">
+        <v>2</v>
+      </c>
+      <c r="E81" s="16"/>
+      <c r="F81" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="G81" s="78">
-        <v>6</v>
-      </c>
-      <c r="H81" s="66"/>
+      <c r="G81" s="18">
+        <v>6</v>
+      </c>
+      <c r="H81" s="50"/>
     </row>
     <row r="82" ht="38.25" customHeight="1">
-      <c r="A82" s="87"/>
-      <c r="B82" s="92"/>
-      <c r="C82" s="93" t="s">
+      <c r="A82" s="58"/>
+      <c r="B82" s="60"/>
+      <c r="C82" s="59" t="s">
         <v>117</v>
       </c>
-      <c r="D82" s="17">
-        <v>2</v>
-      </c>
-      <c r="E82" s="18"/>
-      <c r="F82" s="57"/>
-      <c r="G82" s="79"/>
-      <c r="H82" s="21"/>
+      <c r="D82" s="15">
+        <v>2</v>
+      </c>
+      <c r="E82" s="16"/>
+      <c r="F82" s="38"/>
+      <c r="G82" s="22"/>
+      <c r="H82" s="19"/>
     </row>
     <row r="83" ht="39" customHeight="1">
-      <c r="A83" s="87"/>
-      <c r="B83" s="92"/>
-      <c r="C83" s="93" t="s">
+      <c r="A83" s="58"/>
+      <c r="B83" s="60"/>
+      <c r="C83" s="59" t="s">
         <v>118</v>
       </c>
-      <c r="D83" s="17">
-        <v>2</v>
-      </c>
-      <c r="E83" s="18">
+      <c r="D83" s="15">
+        <v>2</v>
+      </c>
+      <c r="E83" s="16">
         <f>SUM(D81:D83)</f>
         <v>6</v>
       </c>
-      <c r="F83" s="59"/>
-      <c r="G83" s="80"/>
-      <c r="H83" s="70"/>
+      <c r="F83" s="47"/>
+      <c r="G83" s="48"/>
+      <c r="H83" s="53"/>
     </row>
     <row r="84" ht="33.75" customHeight="1">
-      <c r="A84" s="46">
+      <c r="A84" s="43">
         <v>46310</v>
       </c>
-      <c r="B84" s="94" t="s">
+      <c r="B84" s="24" t="s">
         <v>119</v>
       </c>
-      <c r="C84" s="28" t="s">
+      <c r="C84" s="25" t="s">
         <v>120</v>
       </c>
-      <c r="D84" s="28">
-        <v>2</v>
-      </c>
-      <c r="E84" s="29"/>
-      <c r="F84" s="72" t="s">
+      <c r="D84" s="25">
+        <v>2</v>
+      </c>
+      <c r="E84" s="26"/>
+      <c r="F84" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="G84" s="81">
-        <v>6</v>
-      </c>
-      <c r="H84" s="48"/>
+      <c r="G84" s="28">
+        <v>6</v>
+      </c>
+      <c r="H84" s="29"/>
     </row>
     <row r="85" ht="36.75" customHeight="1">
-      <c r="A85" s="46"/>
-      <c r="B85" s="33"/>
-      <c r="C85" s="28" t="s">
+      <c r="A85" s="43"/>
+      <c r="B85" s="30"/>
+      <c r="C85" s="25" t="s">
         <v>121</v>
       </c>
-      <c r="D85" s="28">
-        <v>2</v>
-      </c>
-      <c r="E85" s="34"/>
-      <c r="F85" s="72"/>
-      <c r="G85" s="75"/>
-      <c r="H85" s="50"/>
+      <c r="D85" s="25">
+        <v>2</v>
+      </c>
+      <c r="E85" s="31"/>
+      <c r="F85" s="32"/>
+      <c r="G85" s="33"/>
+      <c r="H85" s="34"/>
     </row>
     <row r="86" ht="33.75" customHeight="1">
-      <c r="A86" s="46"/>
-      <c r="B86" s="38"/>
-      <c r="C86" s="28" t="s">
+      <c r="A86" s="43"/>
+      <c r="B86" s="35"/>
+      <c r="C86" s="25" t="s">
         <v>122</v>
       </c>
-      <c r="D86" s="28">
-        <v>2</v>
-      </c>
-      <c r="E86" s="34">
+      <c r="D86" s="25">
+        <v>2</v>
+      </c>
+      <c r="E86" s="31">
         <f>SUM(D84:D86)</f>
         <v>6</v>
       </c>
-      <c r="F86" s="84"/>
-      <c r="G86" s="76"/>
-      <c r="H86" s="52"/>
+      <c r="F86" s="49"/>
+      <c r="G86" s="44"/>
+      <c r="H86" s="37"/>
     </row>
     <row r="87" ht="38.25" customHeight="1">
-      <c r="A87" s="87">
+      <c r="A87" s="58">
         <v>46311</v>
       </c>
-      <c r="B87" s="91" t="s">
+      <c r="B87" s="60" t="s">
         <v>123</v>
       </c>
-      <c r="C87" s="93" t="s">
+      <c r="C87" s="59" t="s">
         <v>124</v>
       </c>
-      <c r="D87" s="17">
-        <v>2</v>
-      </c>
-      <c r="E87" s="18"/>
-      <c r="F87" s="65" t="s">
+      <c r="D87" s="15">
+        <v>2</v>
+      </c>
+      <c r="E87" s="16"/>
+      <c r="F87" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="G87" s="78">
-        <v>6</v>
-      </c>
-      <c r="H87" s="56"/>
+      <c r="G87" s="18">
+        <v>6</v>
+      </c>
+      <c r="H87" s="39"/>
     </row>
     <row r="88" ht="36" customHeight="1">
-      <c r="A88" s="87"/>
-      <c r="B88" s="92"/>
-      <c r="C88" s="93" t="s">
+      <c r="A88" s="58"/>
+      <c r="B88" s="60"/>
+      <c r="C88" s="59" t="s">
         <v>125</v>
       </c>
-      <c r="D88" s="17">
-        <v>2</v>
-      </c>
-      <c r="E88" s="18"/>
-      <c r="F88" s="67"/>
-      <c r="G88" s="79"/>
-      <c r="H88" s="58"/>
+      <c r="D88" s="15">
+        <v>2</v>
+      </c>
+      <c r="E88" s="16"/>
+      <c r="F88" s="21"/>
+      <c r="G88" s="22"/>
+      <c r="H88" s="40"/>
     </row>
     <row r="89" ht="39.75" customHeight="1">
-      <c r="A89" s="87"/>
-      <c r="B89" s="92"/>
-      <c r="C89" s="89" t="s">
+      <c r="A89" s="58"/>
+      <c r="B89" s="60"/>
+      <c r="C89" s="59" t="s">
         <v>126</v>
       </c>
-      <c r="D89" s="17">
-        <v>2</v>
-      </c>
-      <c r="E89" s="18">
+      <c r="D89" s="15">
+        <v>2</v>
+      </c>
+      <c r="E89" s="16">
         <f>SUM(D87:D89)</f>
         <v>6</v>
       </c>
-      <c r="F89" s="69"/>
-      <c r="G89" s="44"/>
-      <c r="H89" s="61"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="46">
+      <c r="F89" s="52"/>
+      <c r="G89" s="41"/>
+      <c r="H89" s="42"/>
+    </row>
+    <row r="90" ht="28.5">
+      <c r="A90" s="43">
         <v>46314</v>
       </c>
-      <c r="B90" s="95" t="s">
+      <c r="B90" s="57" t="s">
         <v>127</v>
       </c>
-      <c r="C90" s="28" t="s">
+      <c r="C90" s="25" t="s">
         <v>128</v>
       </c>
-      <c r="D90" s="28">
-        <v>2</v>
-      </c>
-      <c r="E90" s="29"/>
-      <c r="F90" s="71" t="s">
+      <c r="D90" s="25">
+        <v>2</v>
+      </c>
+      <c r="E90" s="26"/>
+      <c r="F90" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="G90" s="75">
-        <v>6</v>
-      </c>
-      <c r="H90" s="48"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="46"/>
-      <c r="B91" s="86"/>
-      <c r="C91" s="28" t="s">
+      <c r="G90" s="33">
+        <v>6</v>
+      </c>
+      <c r="H90" s="29"/>
+    </row>
+    <row r="91" ht="28.5">
+      <c r="A91" s="43"/>
+      <c r="B91" s="57"/>
+      <c r="C91" s="25" t="s">
         <v>129</v>
       </c>
-      <c r="D91" s="28">
-        <v>2</v>
-      </c>
-      <c r="E91" s="34"/>
-      <c r="F91" s="72"/>
-      <c r="G91" s="75"/>
-      <c r="H91" s="50"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="46"/>
-      <c r="B92" s="86"/>
-      <c r="C92" s="28" t="s">
+      <c r="D91" s="25">
+        <v>2</v>
+      </c>
+      <c r="E91" s="31"/>
+      <c r="F91" s="32"/>
+      <c r="G91" s="33"/>
+      <c r="H91" s="34"/>
+    </row>
+    <row r="92" ht="28.5">
+      <c r="A92" s="43"/>
+      <c r="B92" s="57"/>
+      <c r="C92" s="25" t="s">
         <v>130</v>
       </c>
-      <c r="D92" s="28">
-        <v>2</v>
-      </c>
-      <c r="E92" s="34">
+      <c r="D92" s="25">
+        <v>2</v>
+      </c>
+      <c r="E92" s="31">
         <f>SUM(D90:D92)</f>
         <v>6</v>
       </c>
-      <c r="F92" s="39"/>
-      <c r="G92" s="76"/>
-      <c r="H92" s="52"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="87">
+      <c r="F92" s="36"/>
+      <c r="G92" s="44"/>
+      <c r="H92" s="37"/>
+    </row>
+    <row r="93" ht="28.5">
+      <c r="A93" s="58">
         <v>46315</v>
       </c>
-      <c r="B93" s="91" t="s">
+      <c r="B93" s="60" t="s">
         <v>131</v>
       </c>
-      <c r="C93" s="93" t="s">
+      <c r="C93" s="59" t="s">
         <v>132</v>
       </c>
-      <c r="D93" s="17">
-        <v>2</v>
-      </c>
-      <c r="E93" s="18"/>
-      <c r="F93" s="54" t="s">
+      <c r="D93" s="15">
+        <v>2</v>
+      </c>
+      <c r="E93" s="16"/>
+      <c r="F93" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="G93" s="78">
-        <v>6</v>
-      </c>
-      <c r="H93" s="56"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="87"/>
-      <c r="B94" s="92"/>
-      <c r="C94" s="93" t="s">
+      <c r="G93" s="18">
+        <v>6</v>
+      </c>
+      <c r="H93" s="39"/>
+    </row>
+    <row r="94" ht="28.5">
+      <c r="A94" s="58"/>
+      <c r="B94" s="60"/>
+      <c r="C94" s="59" t="s">
         <v>133</v>
       </c>
-      <c r="D94" s="17">
-        <v>2</v>
-      </c>
-      <c r="E94" s="18"/>
-      <c r="F94" s="57"/>
-      <c r="G94" s="79"/>
-      <c r="H94" s="58"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="87"/>
-      <c r="B95" s="92"/>
-      <c r="C95" s="93" t="s">
+      <c r="D94" s="15">
+        <v>2</v>
+      </c>
+      <c r="E94" s="16"/>
+      <c r="F94" s="38"/>
+      <c r="G94" s="22"/>
+      <c r="H94" s="40"/>
+    </row>
+    <row r="95" ht="28.5">
+      <c r="A95" s="58"/>
+      <c r="B95" s="60"/>
+      <c r="C95" s="59" t="s">
         <v>134</v>
       </c>
-      <c r="D95" s="17">
-        <v>2</v>
-      </c>
-      <c r="E95" s="18">
+      <c r="D95" s="15">
+        <v>2</v>
+      </c>
+      <c r="E95" s="16">
         <f>SUM(D93:D95)</f>
         <v>6</v>
       </c>
-      <c r="F95" s="74"/>
-      <c r="G95" s="80"/>
-      <c r="H95" s="61"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="46">
+      <c r="F95" s="54"/>
+      <c r="G95" s="48"/>
+      <c r="H95" s="42"/>
+    </row>
+    <row r="96" ht="28.5">
+      <c r="A96" s="43">
         <v>46316</v>
       </c>
-      <c r="B96" s="95" t="s">
+      <c r="B96" s="57" t="s">
         <v>135</v>
       </c>
-      <c r="C96" s="28" t="s">
+      <c r="C96" s="25" t="s">
         <v>136</v>
       </c>
-      <c r="D96" s="28">
-        <v>2</v>
-      </c>
-      <c r="E96" s="29"/>
-      <c r="F96" s="71" t="s">
+      <c r="D96" s="25">
+        <v>2</v>
+      </c>
+      <c r="E96" s="26"/>
+      <c r="F96" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="G96" s="81">
-        <v>6</v>
-      </c>
-      <c r="H96" s="48"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="46"/>
-      <c r="B97" s="86"/>
-      <c r="C97" s="28" t="s">
+      <c r="G96" s="28">
+        <v>6</v>
+      </c>
+      <c r="H96" s="29"/>
+    </row>
+    <row r="97" ht="28.5">
+      <c r="A97" s="43"/>
+      <c r="B97" s="57"/>
+      <c r="C97" s="25" t="s">
         <v>137</v>
       </c>
-      <c r="D97" s="28">
-        <v>2</v>
-      </c>
-      <c r="E97" s="34"/>
-      <c r="F97" s="72"/>
-      <c r="G97" s="75"/>
-      <c r="H97" s="50"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="46"/>
-      <c r="B98" s="86"/>
-      <c r="C98" s="28" t="s">
+      <c r="D97" s="25">
+        <v>2</v>
+      </c>
+      <c r="E97" s="31"/>
+      <c r="F97" s="32"/>
+      <c r="G97" s="33"/>
+      <c r="H97" s="34"/>
+    </row>
+    <row r="98" ht="28.5">
+      <c r="A98" s="43"/>
+      <c r="B98" s="57"/>
+      <c r="C98" s="25" t="s">
         <v>138</v>
       </c>
-      <c r="D98" s="28">
-        <v>2</v>
-      </c>
-      <c r="E98" s="34">
+      <c r="D98" s="25">
+        <v>2</v>
+      </c>
+      <c r="E98" s="31">
         <f>SUM(D96:D98)</f>
         <v>6</v>
       </c>
-      <c r="F98" s="39"/>
-      <c r="G98" s="76"/>
-      <c r="H98" s="52"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="87">
+      <c r="F98" s="36"/>
+      <c r="G98" s="44"/>
+      <c r="H98" s="37"/>
+    </row>
+    <row r="99" ht="28.5">
+      <c r="A99" s="58">
         <v>46317</v>
       </c>
-      <c r="B99" s="91" t="s">
+      <c r="B99" s="60" t="s">
         <v>139</v>
       </c>
-      <c r="C99" s="93" t="s">
+      <c r="C99" s="59" t="s">
         <v>140</v>
       </c>
-      <c r="D99" s="17">
-        <v>2</v>
-      </c>
-      <c r="E99" s="18"/>
-      <c r="F99" s="54" t="s">
+      <c r="D99" s="15">
+        <v>2</v>
+      </c>
+      <c r="E99" s="16"/>
+      <c r="F99" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="G99" s="78">
-        <v>6</v>
-      </c>
-      <c r="H99" s="66"/>
-    </row>
-    <row r="100">
-      <c r="A100" s="87"/>
-      <c r="B100" s="92"/>
-      <c r="C100" s="93" t="s">
+      <c r="G99" s="18">
+        <v>6</v>
+      </c>
+      <c r="H99" s="50"/>
+    </row>
+    <row r="100" ht="28.5">
+      <c r="A100" s="58"/>
+      <c r="B100" s="60"/>
+      <c r="C100" s="59" t="s">
         <v>141</v>
       </c>
-      <c r="D100" s="17">
-        <v>2</v>
-      </c>
-      <c r="E100" s="18"/>
-      <c r="F100" s="57"/>
-      <c r="G100" s="79"/>
-      <c r="H100" s="21"/>
-    </row>
-    <row r="101">
-      <c r="A101" s="87"/>
-      <c r="B101" s="92"/>
-      <c r="C101" s="89" t="s">
+      <c r="D100" s="15">
+        <v>2</v>
+      </c>
+      <c r="E100" s="16"/>
+      <c r="F100" s="38"/>
+      <c r="G100" s="22"/>
+      <c r="H100" s="19"/>
+    </row>
+    <row r="101" ht="28.5">
+      <c r="A101" s="58"/>
+      <c r="B101" s="60"/>
+      <c r="C101" s="59" t="s">
         <v>142</v>
       </c>
-      <c r="D101" s="17">
-        <v>2</v>
-      </c>
-      <c r="E101" s="18">
+      <c r="D101" s="15">
+        <v>2</v>
+      </c>
+      <c r="E101" s="16">
         <f>SUM(D99:D101)</f>
         <v>6</v>
       </c>
-      <c r="F101" s="41"/>
-      <c r="G101" s="44"/>
-      <c r="H101" s="70"/>
-    </row>
-    <row r="102">
-      <c r="A102" s="46">
+      <c r="F101" s="38"/>
+      <c r="G101" s="41"/>
+      <c r="H101" s="53"/>
+    </row>
+    <row r="102" ht="28.5">
+      <c r="A102" s="43">
         <v>46318</v>
       </c>
-      <c r="B102" s="96" t="s">
+      <c r="B102" s="61" t="s">
         <v>143</v>
       </c>
-      <c r="C102" s="28" t="s">
+      <c r="C102" s="25" t="s">
         <v>144</v>
       </c>
-      <c r="D102" s="28">
-        <v>2</v>
-      </c>
-      <c r="E102" s="29"/>
-      <c r="F102" s="47" t="s">
+      <c r="D102" s="25">
+        <v>2</v>
+      </c>
+      <c r="E102" s="26"/>
+      <c r="F102" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="G102" s="82">
-        <v>6</v>
-      </c>
-      <c r="H102" s="48"/>
-    </row>
-    <row r="103">
-      <c r="A103" s="46"/>
-      <c r="B103" s="97"/>
-      <c r="C103" s="28" t="s">
+      <c r="G102" s="33">
+        <v>6</v>
+      </c>
+      <c r="H102" s="29"/>
+    </row>
+    <row r="103" ht="28.5">
+      <c r="A103" s="43"/>
+      <c r="B103" s="61"/>
+      <c r="C103" s="25" t="s">
         <v>145</v>
       </c>
-      <c r="D103" s="28">
-        <v>2</v>
-      </c>
-      <c r="E103" s="34"/>
-      <c r="F103" s="49"/>
-      <c r="G103" s="83"/>
-      <c r="H103" s="50"/>
-    </row>
-    <row r="104">
-      <c r="A104" s="46"/>
-      <c r="B104" s="97"/>
-      <c r="C104" s="28" t="s">
+      <c r="D103" s="25">
+        <v>2</v>
+      </c>
+      <c r="E103" s="31"/>
+      <c r="F103" s="32"/>
+      <c r="G103" s="33"/>
+      <c r="H103" s="34"/>
+    </row>
+    <row r="104" ht="28.5">
+      <c r="A104" s="43"/>
+      <c r="B104" s="61"/>
+      <c r="C104" s="25" t="s">
         <v>146</v>
       </c>
-      <c r="D104" s="28">
-        <v>2</v>
-      </c>
-      <c r="E104" s="34">
+      <c r="D104" s="25">
+        <v>2</v>
+      </c>
+      <c r="E104" s="31">
         <f>SUM(D102:D104)</f>
         <v>6</v>
       </c>
-      <c r="F104" s="39"/>
-      <c r="G104" s="85"/>
-      <c r="H104" s="52"/>
-    </row>
-    <row r="105">
-      <c r="A105" s="98">
+      <c r="F104" s="36"/>
+      <c r="G104" s="44"/>
+      <c r="H104" s="37"/>
+    </row>
+    <row r="105" ht="28.5">
+      <c r="A105" s="62">
         <v>46321</v>
       </c>
-      <c r="B105" s="99" t="s">
+      <c r="B105" s="63" t="s">
         <v>147</v>
       </c>
-      <c r="C105" s="93" t="s">
+      <c r="C105" s="59" t="s">
         <v>148</v>
       </c>
-      <c r="D105" s="17">
-        <v>2</v>
-      </c>
-      <c r="E105" s="18"/>
-      <c r="F105" s="54" t="s">
+      <c r="D105" s="15">
+        <v>2</v>
+      </c>
+      <c r="E105" s="16"/>
+      <c r="F105" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="G105" s="78">
-        <v>6</v>
-      </c>
-      <c r="H105" s="56"/>
-    </row>
-    <row r="106">
-      <c r="A106" s="87"/>
-      <c r="B106" s="92"/>
-      <c r="C106" s="93" t="s">
+      <c r="G105" s="18">
+        <v>6</v>
+      </c>
+      <c r="H105" s="39"/>
+    </row>
+    <row r="106" ht="28.5">
+      <c r="A106" s="58"/>
+      <c r="B106" s="60"/>
+      <c r="C106" s="59" t="s">
         <v>149</v>
       </c>
-      <c r="D106" s="17">
-        <v>2</v>
-      </c>
-      <c r="E106" s="18"/>
-      <c r="F106" s="57"/>
-      <c r="G106" s="79"/>
-      <c r="H106" s="58"/>
-    </row>
-    <row r="107">
-      <c r="A107" s="100"/>
-      <c r="B107" s="101"/>
-      <c r="C107" s="93" t="s">
+      <c r="D106" s="15">
+        <v>2</v>
+      </c>
+      <c r="E106" s="16"/>
+      <c r="F106" s="38"/>
+      <c r="G106" s="22"/>
+      <c r="H106" s="40"/>
+    </row>
+    <row r="107" ht="28.5">
+      <c r="A107" s="64"/>
+      <c r="B107" s="65"/>
+      <c r="C107" s="59" t="s">
         <v>150</v>
       </c>
-      <c r="D107" s="17">
-        <v>2</v>
-      </c>
-      <c r="E107" s="18">
+      <c r="D107" s="15">
+        <v>2</v>
+      </c>
+      <c r="E107" s="16">
         <f>SUM(D105:D107)</f>
         <v>6</v>
       </c>
-      <c r="F107" s="74"/>
-      <c r="G107" s="80"/>
-      <c r="H107" s="61"/>
-    </row>
-    <row r="108" ht="17">
-      <c r="A108" s="26">
+      <c r="F107" s="54"/>
+      <c r="G107" s="48"/>
+      <c r="H107" s="42"/>
+    </row>
+    <row r="108" ht="28.5">
+      <c r="A108" s="24">
         <v>46322</v>
       </c>
-      <c r="B108" s="102" t="s">
+      <c r="B108" s="66" t="s">
         <v>151</v>
       </c>
-      <c r="C108" s="28" t="s">
+      <c r="C108" s="25" t="s">
         <v>152</v>
       </c>
-      <c r="D108" s="28">
-        <v>2</v>
-      </c>
-      <c r="E108" s="29"/>
-      <c r="F108" s="71" t="s">
+      <c r="D108" s="25">
+        <v>2</v>
+      </c>
+      <c r="E108" s="26"/>
+      <c r="F108" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="G108" s="81">
-        <v>6</v>
-      </c>
-      <c r="H108" s="48"/>
-    </row>
-    <row r="109" ht="34">
-      <c r="A109" s="46"/>
-      <c r="B109" s="86"/>
-      <c r="C109" s="28" t="s">
+      <c r="G108" s="28">
+        <v>6</v>
+      </c>
+      <c r="H108" s="29"/>
+    </row>
+    <row r="109" ht="28.5">
+      <c r="A109" s="43"/>
+      <c r="B109" s="57"/>
+      <c r="C109" s="25" t="s">
         <v>153</v>
       </c>
-      <c r="D109" s="28">
-        <v>2</v>
-      </c>
-      <c r="E109" s="34"/>
-      <c r="F109" s="72"/>
-      <c r="G109" s="75"/>
-      <c r="H109" s="50"/>
-    </row>
-    <row r="110" ht="17">
-      <c r="A110" s="38"/>
-      <c r="B110" s="103"/>
-      <c r="C110" s="28" t="s">
+      <c r="D109" s="25">
+        <v>2</v>
+      </c>
+      <c r="E109" s="31"/>
+      <c r="F109" s="32"/>
+      <c r="G109" s="33"/>
+      <c r="H109" s="34"/>
+    </row>
+    <row r="110" ht="28.5">
+      <c r="A110" s="35"/>
+      <c r="B110" s="67"/>
+      <c r="C110" s="25" t="s">
         <v>154</v>
       </c>
-      <c r="D110" s="28">
-        <v>2</v>
-      </c>
-      <c r="E110" s="34">
+      <c r="D110" s="25">
+        <v>2</v>
+      </c>
+      <c r="E110" s="31">
         <f>SUM(D108:D110)</f>
         <v>6</v>
       </c>
-      <c r="F110" s="39"/>
-      <c r="G110" s="76"/>
-      <c r="H110" s="52"/>
-    </row>
-    <row r="111">
-      <c r="A111" s="104">
+      <c r="F110" s="36"/>
+      <c r="G110" s="44"/>
+      <c r="H110" s="37"/>
+    </row>
+    <row r="111" ht="28.5">
+      <c r="A111" s="68">
         <v>46323</v>
       </c>
-      <c r="B111" s="99" t="s">
+      <c r="B111" s="63" t="s">
         <v>155</v>
       </c>
-      <c r="C111" s="93" t="s">
+      <c r="C111" s="59" t="s">
         <v>156</v>
       </c>
-      <c r="D111" s="17">
-        <v>2</v>
-      </c>
-      <c r="E111" s="18"/>
-      <c r="F111" s="54" t="s">
+      <c r="D111" s="15">
+        <v>2</v>
+      </c>
+      <c r="E111" s="16"/>
+      <c r="F111" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="G111" s="78">
-        <v>6</v>
-      </c>
-      <c r="H111" s="56"/>
-    </row>
-    <row r="112">
-      <c r="A112" s="105"/>
-      <c r="B112" s="92"/>
-      <c r="C112" s="93" t="s">
+      <c r="G111" s="18">
+        <v>6</v>
+      </c>
+      <c r="H111" s="39"/>
+    </row>
+    <row r="112" ht="28.5">
+      <c r="A112" s="69"/>
+      <c r="B112" s="60"/>
+      <c r="C112" s="59" t="s">
         <v>157</v>
       </c>
-      <c r="D112" s="17">
-        <v>2</v>
-      </c>
-      <c r="E112" s="18"/>
-      <c r="F112" s="57"/>
-      <c r="G112" s="79"/>
-      <c r="H112" s="58"/>
-    </row>
-    <row r="113">
-      <c r="A113" s="106"/>
-      <c r="B113" s="101"/>
-      <c r="C113" s="93" t="s">
+      <c r="D112" s="15">
+        <v>2</v>
+      </c>
+      <c r="E112" s="16"/>
+      <c r="F112" s="38"/>
+      <c r="G112" s="22"/>
+      <c r="H112" s="40"/>
+    </row>
+    <row r="113" ht="28.5">
+      <c r="A113" s="70"/>
+      <c r="B113" s="65"/>
+      <c r="C113" s="59" t="s">
         <v>158</v>
       </c>
-      <c r="D113" s="17">
-        <v>2</v>
-      </c>
-      <c r="E113" s="18">
+      <c r="D113" s="15">
+        <v>2</v>
+      </c>
+      <c r="E113" s="16">
         <f>SUM(D111:D113)</f>
         <v>6</v>
       </c>
-      <c r="F113" s="41"/>
-      <c r="G113" s="44"/>
-      <c r="H113" s="107"/>
-    </row>
-    <row r="114">
-      <c r="A114" s="108">
+      <c r="F113" s="38"/>
+      <c r="G113" s="41"/>
+      <c r="H113" s="40"/>
+    </row>
+    <row r="114" ht="28.5">
+      <c r="A114" s="71">
         <v>46324</v>
       </c>
-      <c r="B114" s="109" t="s">
+      <c r="B114" s="27" t="s">
         <v>159</v>
       </c>
-      <c r="C114" s="28" t="s">
+      <c r="C114" s="25" t="s">
         <v>160</v>
       </c>
-      <c r="D114" s="28">
-        <v>2</v>
-      </c>
-      <c r="E114" s="29"/>
-      <c r="F114" s="47" t="s">
+      <c r="D114" s="25">
+        <v>2</v>
+      </c>
+      <c r="E114" s="26"/>
+      <c r="F114" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="G114" s="75">
-        <v>6</v>
-      </c>
-      <c r="H114" s="32"/>
-    </row>
-    <row r="115">
-      <c r="A115" s="110"/>
-      <c r="B115" s="97"/>
-      <c r="C115" s="28" t="s">
+      <c r="G114" s="33">
+        <v>6</v>
+      </c>
+      <c r="H114" s="29"/>
+    </row>
+    <row r="115" ht="28.5">
+      <c r="A115" s="72"/>
+      <c r="B115" s="61"/>
+      <c r="C115" s="25" t="s">
         <v>161</v>
       </c>
-      <c r="D115" s="28">
-        <v>2</v>
-      </c>
-      <c r="E115" s="34"/>
-      <c r="F115" s="49"/>
-      <c r="G115" s="75"/>
-      <c r="H115" s="37"/>
-    </row>
-    <row r="116">
-      <c r="A116" s="111"/>
-      <c r="B116" s="64"/>
-      <c r="C116" s="28" t="s">
+      <c r="D115" s="25">
+        <v>2</v>
+      </c>
+      <c r="E115" s="31"/>
+      <c r="F115" s="32"/>
+      <c r="G115" s="33"/>
+      <c r="H115" s="34"/>
+    </row>
+    <row r="116" ht="28.5">
+      <c r="A116" s="73"/>
+      <c r="B116" s="49"/>
+      <c r="C116" s="25" t="s">
         <v>162</v>
       </c>
-      <c r="D116" s="28">
-        <v>2</v>
-      </c>
-      <c r="E116" s="34">
+      <c r="D116" s="25">
+        <v>2</v>
+      </c>
+      <c r="E116" s="31">
         <f>SUM(D114:D116)</f>
         <v>6</v>
       </c>
-      <c r="F116" s="39"/>
-      <c r="G116" s="76"/>
-      <c r="H116" s="40"/>
-    </row>
-    <row r="117">
-      <c r="A117" s="104">
+      <c r="F116" s="36"/>
+      <c r="G116" s="44"/>
+      <c r="H116" s="37"/>
+    </row>
+    <row r="117" ht="28.5">
+      <c r="A117" s="68">
         <v>46325</v>
       </c>
-      <c r="B117" s="99" t="s">
+      <c r="B117" s="63" t="s">
         <v>163</v>
       </c>
-      <c r="C117" s="93" t="s">
+      <c r="C117" s="59" t="s">
         <v>164</v>
       </c>
-      <c r="D117" s="17">
-        <v>2</v>
-      </c>
-      <c r="E117" s="18"/>
-      <c r="F117" s="54" t="s">
+      <c r="D117" s="15">
+        <v>2</v>
+      </c>
+      <c r="E117" s="16"/>
+      <c r="F117" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="G117" s="78">
-        <v>6</v>
-      </c>
-      <c r="H117" s="42"/>
-    </row>
-    <row r="118">
-      <c r="A118" s="105"/>
-      <c r="B118" s="92"/>
-      <c r="C118" s="89" t="s">
+      <c r="G117" s="18">
+        <v>6</v>
+      </c>
+      <c r="H117" s="39"/>
+    </row>
+    <row r="118" ht="28.5">
+      <c r="A118" s="69"/>
+      <c r="B118" s="60"/>
+      <c r="C118" s="59" t="s">
         <v>165</v>
       </c>
-      <c r="D118" s="17">
-        <v>2</v>
-      </c>
-      <c r="E118" s="18"/>
-      <c r="F118" s="57"/>
-      <c r="G118" s="79"/>
-      <c r="H118" s="43"/>
-    </row>
-    <row r="119">
-      <c r="A119" s="106"/>
-      <c r="B119" s="101"/>
-      <c r="C119" s="89" t="s">
+      <c r="D118" s="15">
+        <v>2</v>
+      </c>
+      <c r="E118" s="16"/>
+      <c r="F118" s="38"/>
+      <c r="G118" s="22"/>
+      <c r="H118" s="40"/>
+    </row>
+    <row r="119" ht="28.5">
+      <c r="A119" s="70"/>
+      <c r="B119" s="65"/>
+      <c r="C119" s="59" t="s">
         <v>166</v>
       </c>
-      <c r="D119" s="17">
-        <v>2</v>
-      </c>
-      <c r="E119" s="18">
+      <c r="D119" s="15">
+        <v>2</v>
+      </c>
+      <c r="E119" s="16">
         <f>SUM(D117:D119)</f>
         <v>6</v>
       </c>
-      <c r="F119" s="74"/>
-      <c r="G119" s="80"/>
-      <c r="H119" s="45"/>
-    </row>
-    <row r="120">
-      <c r="A120" s="108">
+      <c r="F119" s="54"/>
+      <c r="G119" s="48"/>
+      <c r="H119" s="42"/>
+    </row>
+    <row r="120" ht="28.5">
+      <c r="A120" s="71">
         <v>46330</v>
       </c>
-      <c r="B120" s="102" t="s">
+      <c r="B120" s="66" t="s">
         <v>167</v>
       </c>
-      <c r="C120" s="28" t="s">
+      <c r="C120" s="25" t="s">
         <v>168</v>
       </c>
-      <c r="D120" s="28">
-        <v>2</v>
-      </c>
-      <c r="E120" s="29"/>
-      <c r="F120" s="71" t="s">
+      <c r="D120" s="25">
+        <v>2</v>
+      </c>
+      <c r="E120" s="26"/>
+      <c r="F120" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="G120" s="81">
-        <v>6</v>
-      </c>
-      <c r="H120" s="37"/>
-    </row>
-    <row r="121">
-      <c r="A121" s="110"/>
-      <c r="B121" s="86"/>
-      <c r="C121" s="28" t="s">
+      <c r="G120" s="28">
+        <v>6</v>
+      </c>
+      <c r="H120" s="34"/>
+    </row>
+    <row r="121" ht="28.5">
+      <c r="A121" s="72"/>
+      <c r="B121" s="57"/>
+      <c r="C121" s="25" t="s">
         <v>169</v>
       </c>
-      <c r="D121" s="28">
-        <v>2</v>
-      </c>
-      <c r="E121" s="34"/>
-      <c r="F121" s="72"/>
-      <c r="G121" s="75"/>
-      <c r="H121" s="37"/>
-    </row>
-    <row r="122">
-      <c r="A122" s="111"/>
-      <c r="B122" s="103"/>
-      <c r="C122" s="28" t="s">
+      <c r="D121" s="25">
+        <v>2</v>
+      </c>
+      <c r="E121" s="31"/>
+      <c r="F121" s="32"/>
+      <c r="G121" s="33"/>
+      <c r="H121" s="34"/>
+    </row>
+    <row r="122" ht="28.5">
+      <c r="A122" s="73"/>
+      <c r="B122" s="67"/>
+      <c r="C122" s="25" t="s">
         <v>170</v>
       </c>
-      <c r="D122" s="28">
-        <v>2</v>
-      </c>
-      <c r="E122" s="34">
+      <c r="D122" s="25">
+        <v>2</v>
+      </c>
+      <c r="E122" s="31">
         <f>SUM(D120:D122)</f>
         <v>6</v>
       </c>
-      <c r="F122" s="39"/>
-      <c r="G122" s="76"/>
-      <c r="H122" s="37"/>
-    </row>
-    <row r="123">
-      <c r="A123" s="98">
+      <c r="F122" s="36"/>
+      <c r="G122" s="44"/>
+      <c r="H122" s="34"/>
+    </row>
+    <row r="123" ht="28.5">
+      <c r="A123" s="62">
         <v>46331</v>
       </c>
-      <c r="B123" s="99" t="s">
+      <c r="B123" s="63" t="s">
         <v>171</v>
       </c>
-      <c r="C123" s="89" t="s">
+      <c r="C123" s="59" t="s">
         <v>172</v>
       </c>
-      <c r="D123" s="17">
-        <v>2</v>
-      </c>
-      <c r="E123" s="18"/>
-      <c r="F123" s="54" t="s">
+      <c r="D123" s="15">
+        <v>2</v>
+      </c>
+      <c r="E123" s="16"/>
+      <c r="F123" s="46" t="s">
         <v>20</v>
       </c>
-      <c r="G123" s="78">
-        <v>6</v>
-      </c>
-      <c r="H123" s="42"/>
-    </row>
-    <row r="124">
-      <c r="A124" s="87"/>
-      <c r="B124" s="92"/>
-      <c r="C124" s="89" t="s">
+      <c r="G123" s="18">
+        <v>6</v>
+      </c>
+      <c r="H123" s="39"/>
+    </row>
+    <row r="124" ht="28.5">
+      <c r="A124" s="58"/>
+      <c r="B124" s="60"/>
+      <c r="C124" s="59" t="s">
         <v>173</v>
       </c>
-      <c r="D124" s="17">
-        <v>2</v>
-      </c>
-      <c r="E124" s="18"/>
-      <c r="F124" s="57"/>
-      <c r="G124" s="79"/>
-      <c r="H124" s="43"/>
-    </row>
-    <row r="125">
-      <c r="A125" s="100"/>
-      <c r="B125" s="101"/>
-      <c r="C125" s="89" t="s">
+      <c r="D124" s="15">
+        <v>2</v>
+      </c>
+      <c r="E124" s="16"/>
+      <c r="F124" s="38"/>
+      <c r="G124" s="22"/>
+      <c r="H124" s="40"/>
+    </row>
+    <row r="125" ht="28.5">
+      <c r="A125" s="64"/>
+      <c r="B125" s="65"/>
+      <c r="C125" s="59" t="s">
         <v>174</v>
       </c>
-      <c r="D125" s="17">
-        <v>2</v>
-      </c>
-      <c r="E125" s="18">
+      <c r="D125" s="15">
+        <v>2</v>
+      </c>
+      <c r="E125" s="16">
         <f>SUM(D123:D125)</f>
         <v>6</v>
       </c>
-      <c r="F125" s="59"/>
-      <c r="G125" s="44"/>
-      <c r="H125" s="45"/>
-    </row>
-    <row r="126">
-      <c r="A126" s="26">
+      <c r="F125" s="47"/>
+      <c r="G125" s="41"/>
+      <c r="H125" s="42"/>
+    </row>
+    <row r="126" ht="28.5">
+      <c r="A126" s="24">
         <v>46332</v>
       </c>
-      <c r="B126" s="109" t="s">
+      <c r="B126" s="27" t="s">
         <v>175</v>
       </c>
-      <c r="C126" s="27" t="s">
+      <c r="C126" s="25" t="s">
         <v>172</v>
       </c>
-      <c r="D126" s="28">
-        <v>2</v>
-      </c>
-      <c r="E126" s="29"/>
-      <c r="F126" s="62" t="s">
+      <c r="D126" s="25">
+        <v>2</v>
+      </c>
+      <c r="E126" s="26"/>
+      <c r="F126" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="G126" s="36">
-        <v>6</v>
-      </c>
-      <c r="H126" s="37"/>
-    </row>
-    <row r="127">
-      <c r="A127" s="46"/>
-      <c r="B127" s="97"/>
-      <c r="C127" s="27" t="s">
+      <c r="G126" s="33">
+        <v>6</v>
+      </c>
+      <c r="H126" s="34"/>
+    </row>
+    <row r="127" ht="28.5">
+      <c r="A127" s="43"/>
+      <c r="B127" s="61"/>
+      <c r="C127" s="25" t="s">
         <v>173</v>
       </c>
-      <c r="D127" s="28">
-        <v>2</v>
-      </c>
-      <c r="E127" s="34"/>
-      <c r="F127" s="35"/>
-      <c r="G127" s="36"/>
-      <c r="H127" s="37"/>
-    </row>
-    <row r="128">
-      <c r="A128" s="38"/>
-      <c r="B128" s="64"/>
-      <c r="C128" s="27" t="s">
+      <c r="D127" s="25">
+        <v>2</v>
+      </c>
+      <c r="E127" s="31"/>
+      <c r="F127" s="32"/>
+      <c r="G127" s="33"/>
+      <c r="H127" s="34"/>
+    </row>
+    <row r="128" ht="28.5">
+      <c r="A128" s="35"/>
+      <c r="B128" s="49"/>
+      <c r="C128" s="25" t="s">
         <v>176</v>
       </c>
-      <c r="D128" s="28">
-        <v>2</v>
-      </c>
-      <c r="E128" s="34">
+      <c r="D128" s="25">
+        <v>2</v>
+      </c>
+      <c r="E128" s="31">
         <f>SUM(D126:D128)</f>
         <v>6</v>
       </c>
-      <c r="F128" s="64"/>
-      <c r="G128" s="51"/>
-      <c r="H128" s="40"/>
+      <c r="F128" s="49"/>
+      <c r="G128" s="44"/>
+      <c r="H128" s="37"/>
     </row>
     <row r="129">
       <c r="A129" s="1"/>
-      <c r="B129" s="112"/>
+      <c r="B129" s="74"/>
       <c r="C129" s="3"/>
       <c r="D129" s="3"/>
       <c r="E129" s="4"/>
@@ -4252,29 +3934,29 @@
     </row>
     <row r="130">
       <c r="A130" s="1"/>
-      <c r="B130" s="112"/>
+      <c r="B130" s="74"/>
       <c r="C130" s="1"/>
-      <c r="D130" s="113"/>
-      <c r="E130" s="114"/>
+      <c r="D130" s="75"/>
+      <c r="E130" s="76"/>
       <c r="F130" s="4"/>
-      <c r="G130" s="115"/>
+      <c r="G130" s="77"/>
       <c r="H130" s="5"/>
     </row>
     <row r="131">
       <c r="A131" s="1"/>
-      <c r="B131" s="112"/>
+      <c r="B131" s="74"/>
       <c r="C131" s="3"/>
-      <c r="D131" s="116" t="s">
+      <c r="D131" s="78" t="s">
         <v>177</v>
       </c>
-      <c r="E131" s="117">
+      <c r="E131" s="79">
         <f>SUM(E9:E128)</f>
         <v>240</v>
       </c>
-      <c r="F131" s="118" t="s">
+      <c r="F131" s="80" t="s">
         <v>178</v>
       </c>
-      <c r="G131" s="119">
+      <c r="G131" s="81">
         <f>SUM(G9:G128)</f>
         <v>240</v>
       </c>
@@ -4282,17 +3964,17 @@
     </row>
     <row r="132">
       <c r="A132" s="1"/>
-      <c r="B132" s="112"/>
+      <c r="B132" s="74"/>
       <c r="C132" s="3"/>
       <c r="D132" s="3"/>
       <c r="E132" s="4"/>
-      <c r="F132" s="120"/>
-      <c r="G132" s="121"/>
+      <c r="F132" s="82"/>
+      <c r="G132" s="83"/>
       <c r="H132" s="5"/>
     </row>
     <row r="133">
       <c r="A133" s="1"/>
-      <c r="B133" s="112"/>
+      <c r="B133" s="74"/>
       <c r="C133" s="3"/>
       <c r="D133" s="3"/>
       <c r="E133" s="4"/>
@@ -4301,7 +3983,7 @@
     </row>
     <row r="134">
       <c r="A134" s="1"/>
-      <c r="B134" s="112"/>
+      <c r="B134" s="74"/>
       <c r="C134" s="3"/>
       <c r="D134" s="3"/>
       <c r="E134" s="4"/>
@@ -4310,7 +3992,7 @@
     </row>
     <row r="135">
       <c r="A135" s="1"/>
-      <c r="B135" s="112"/>
+      <c r="B135" s="74"/>
       <c r="C135" s="3"/>
       <c r="D135" s="3"/>
       <c r="E135" s="4"/>
@@ -4319,7 +4001,7 @@
     </row>
     <row r="136">
       <c r="A136" s="1"/>
-      <c r="B136" s="112"/>
+      <c r="B136" s="74"/>
       <c r="C136" s="3"/>
       <c r="D136" s="3"/>
       <c r="E136" s="4"/>

</xml_diff>